<commit_message>
Update WMP gap register to Rev 3: join model, shop-floor MFA, licensing
Incorporates WMP's latest answers: pure Entra ID join (G-09 resolved,
with follow-through to simplify CA policy 3 and remove Seamless SSO;
cascades into the sync-design row - PHS alone), shop-floor MFA =
Authenticator with YubiKey fallback (G-11 trimmed to registration
logistics), and the full 150-user licensing plan recorded (15 G5 / 55
Business Premium tier + Defender-Purview suite / 80 F3 + F5 S&C, Teams
Phone x55). G-07 resolved (Entra P2 arrives via the SKU mix); remaining
G-06 question flags that the 55-seat Business Premium line carries no
GCCH marker and needs AOS-G partner verification. 41 open (27 High / 14
Medium), 23 resolved; recalculated clean.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01D9SFx2c7BjowTfENYrpiQo
</commit_message>
<xml_diff>
--- a/deliverables/WMP/WMP__Solution_Design_Gap_Register__20260824.xlsx
+++ b/deliverables/WMP/WMP__Solution_Design_Gap_Register__20260824.xlsx
@@ -13,8 +13,8 @@
     <sheet name="Resolved Decisions" sheetId="3" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
-    <definedName function="false" hidden="true" localSheetId="1" name="_xlnm._FilterDatabase" vbProcedure="false">'Gap Register'!$A$1:$K$44</definedName>
-    <definedName function="false" hidden="true" localSheetId="2" name="_xlnm._FilterDatabase" vbProcedure="false">'Resolved Decisions'!$A$1:$E$22</definedName>
+    <definedName function="false" hidden="true" localSheetId="1" name="_xlnm._FilterDatabase" vbProcedure="false">'Gap Register'!$A$1:$K$42</definedName>
+    <definedName function="false" hidden="true" localSheetId="2" name="_xlnm._FilterDatabase" vbProcedure="false">'Resolved Decisions'!$A$1:$E$24</definedName>
   </definedNames>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -26,12 +26,12 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="613" uniqueCount="385">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="602" uniqueCount="382">
   <si>
     <t xml:space="preserve">WMP Solution Design — Inputs &amp; Decisions Gap Register</t>
   </si>
   <si>
-    <t xml:space="preserve">Rev 2 — updated 8/24/2026 with WMP's responses. Open questions only; resolved decisions on the 'Resolved Decisions' sheet.</t>
+    <t xml:space="preserve">Rev 3 — updated 8/24/2026: join model, shop-floor MFA, and the licensing plan incorporated. Open questions only; resolved decisions on the 'Resolved Decisions' sheet.</t>
   </si>
   <si>
     <t xml:space="preserve">Wisconsin Metal Parts — Microsoft GCC High Migration (CMMC 2.0 Level 2)  |  Prepared by Essendis</t>
@@ -40,7 +40,7 @@
     <t xml:space="preserve">Purpose</t>
   </si>
   <si>
-    <t xml:space="preserve">The register now carries only the questions still open after WMP's first review pass. Each answered row moved to the Resolved Decisions sheet with its follow-through (the design-doc edit or configuration action it drives). Partially answered rows remain here with the decided part recorded and only the outstanding questions listed.</t>
+    <t xml:space="preserve">The register carries only the questions still open after WMP's review passes. Answered rows live on the Resolved Decisions sheet with the follow-through each decision drives (design-doc edit or configuration action). Partially answered rows remain here with the decided part recorded and only the outstanding questions listed.</t>
   </si>
   <si>
     <t xml:space="preserve">How to read the register</t>
@@ -270,34 +270,22 @@
     <t xml:space="preserve">Half the controls in this design are SKU-dependent (PIM, risk policies, Defender for Endpoint, Purview labelling/DLP, audit retention); costing and configuration both stall until the SKU is fixed.</t>
   </si>
   <si>
-    <t xml:space="preserve">Provide the licensing quote (promised, not yet received) and confirm the final SKU mix per persona from it.
-Confirm the quote covers: Entra ID P2 (G-07), Defender for Endpoint P2 (G-28), Endpoint DLP (G-58), Teams Phone.
+    <t xml:space="preserve">Confirm with the AOS-G partner that the 55-seat tier is a GCC High offering: the quote line reads 'M365 Business Premium' with no GCCH marker, and Business Premium has no native GCC High variant — verify what the paired 'BP Defender Purview Suite GCCH' actually delivers, specifically Entra ID P2 and Endpoint DLP entitlements for those 55 users.
 Who buys AvePoint Fly, ForensIT, and CallTower seats — WMP directly or through Essendis?
 How long do commercial-tenant licences overlap GCC High, and is the overlap budgeted?</t>
   </si>
   <si>
-    <t xml:space="preserve">WMP (8/24): I'll attach licensing quote</t>
+    <t xml:space="preserve">WMP (8/24) licensing plan received:
+M365 G5 FUSL GCCH x15 (ADD-99035-COMM)
+M365 Business Premium x55 (AAD-59343-COMM-2)
+BP Defender Purview Suite GCCH x55 (AAV-01856-COMM-2)
+Teams Phone Standard GCCH x55 (RFT-00001-COMM)
+M365 F3 GCCH x80 (AAA-99952-COMM)
+M365 F5 Security + Compliance GCCH Add-on x80 (91Q-00003-COMM)
+= 150 users: 15 G5 / 55 BP tier / 80 F3 + F5 S&amp;C.</t>
   </si>
   <si>
     <t xml:space="preserve">New section: M365 Design &gt; Licensing</t>
-  </si>
-  <si>
-    <t xml:space="preserve">G-07</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Entra ID P1 vs P2 is unresolved in the document — CA policy 7 says "Requires Entra ID P2" and policy 8 is titled "If P2". The dependency is broader than those two policies: PIM (used in two sections and Deployment phase 1) and access reviews also require P2.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">If only P1 is purchased, three commitments in the design collapse at once: risk-based CA, PIM just-in-time elevation, and access reviews — all of which the RPO is likely to map to AC.L2-3.1.5/3.1.7 evidence.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Entra ID P2 is confirmed in scope — decide the vehicle: included in the base G-SKU or purchased as an add-on (resolve with the G-06 quote).</t>
-  </si>
-  <si>
-    <t xml:space="preserve">WMP (8/24): Included in Sku or as add-on, but not decided which.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Baseline Security &gt; Conditional Access (policies 7 and 8); PIM sections</t>
   </si>
   <si>
     <t xml:space="preserve">G-08</t>
@@ -312,39 +300,17 @@
     <t xml:space="preserve">Sequence the re-point: when does sync cut from the commercial tenant to GCC High relative to the cutover event, and what is the sign-in impact during the gap?
 How are GCC High objects matched to migrated mailboxes (sourceAnchor / ms-DS-ConsistencyGuid vs UPN) so mail lands on the right identities?
 Sync scope: which OUs and object types, and is SSPR password writeback enabled?
-Final sign-in method: PHS alone, or PHS plus Seamless SSO (which only benefits the domain-joined devices WBS 7 retires)?
 Which password policy governs users — on-premises AD or the Appendix A Entra policy (the appendix note citing 'Entra ID Domain Services' appears to be an error)?
 Break-fix: staging server, or a documented rebuild plan if sync fails mid-migration?</t>
   </si>
   <si>
-    <t xml:space="preserve">WMP (8/24): repointing sync to gcch</t>
+    <t xml:space="preserve">WMP (8/24): repointing sync to gcch
+Pure Entra ID join decided (G-09): sign-in is PHS alone; Seamless SSO drops out.</t>
   </si>
   <si>
     <t xml:space="preserve">New section: M365 Design &gt; Hybrid Identity (Entra ID Connect); Appendix A</t>
   </si>
   <si>
-    <t xml:space="preserve">G-09</t>
-  </si>
-  <si>
-    <t xml:space="preserve">The device join model contradicts itself. CA policy 3 is "Require Compliant or Hybrid-Joined Device" and Baseline Security specifies Seamless SSO (an on-premises-domain feature), while WBS 7 disjoins every Windows endpoint from AD, Entra-ID-joins it, and retires GPO.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Join type determines Conditional Access grant wording, how devices authenticate to on-premises resources, and whether GPO or Intune is authoritative — shipping both models guarantees a lockout or an unmanaged fleet at go-live.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Is the end state Entra ID join (cloud-only, per WBS 7) or Entra hybrid join — and is hybrid join even the intent given GPO retirement?
-If Entra ID join is the answer, should CA policy 3's grant be simplified to "require compliant device", and should the Seamless SSO section be removed?
-During the migration window, will both join states coexist — and does the CA device grant tolerate that?
-WBS 1.3.2 records "hybrid join confirmed feasible; departure from prior vendor guidance" — is that still the agreed position, or has it been superseded by the Modern Workspace approach?</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Known from WBS sheet 7: all Windows endpoints are disjoined from AD, Entra ID joined, auto-enrolled in Intune, and GPOs are retired. The design text predates this and should be aligned to a cloud-native join model.
-Signals from WMP's other responses point to pure Entra ID join: G-23 replaces the domain-GUID sync restriction with tenant ID, and G-26 reports no Kerberos-dependent applications. Needs the explicit decision.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Baseline Security &gt; Single Sign-On; CA policy 3; Deployment Approach 5</t>
-  </si>
-  <si>
     <t xml:space="preserve">G-11</t>
   </si>
   <si>
@@ -354,13 +320,13 @@
     <t xml:space="preserve">Authenticator push is not phishing-resistant, so the admin policy as written cannot be satisfied; and NIST SP 800-171 3.5.3 requires MFA for local as well as network access to privileged accounts — which shop-floor workstations cannot meet with a phone-only method.</t>
   </si>
   <si>
-    <t xml:space="preserve">Admins decided: passkey in Authenticator or YubiKey — confirm CA policies 2/4 use the phishing-resistant authentication strength, and who buys/enrols YubiKeys.
-Shop-floor and phone-less users: which factor — FIDO2 keys, Windows Hello for Business, or an issued device?
-Pre-cutover registration for ~150 users: Temporary Access Pass, a registration CA policy, or supervised on-site sessions per site?
+    <t xml:space="preserve">Pre-cutover MFA registration logistics for ~150 users: Temporary Access Pass, a registration-only CA policy, or supervised on-site sessions per site?
+How many YubiKeys are needed for fallback users, and who purchases and enrols them?
 Is SMS/voice MFA explicitly disallowed?</t>
   </si>
   <si>
-    <t xml:space="preserve">WMP (8/24): Admins should use passkey in authenticator or Yubikey</t>
+    <t xml:space="preserve">WMP (8/24): Admins should use passkey in authenticator or Yubikey
+WMP (8/24): shop-floor MFA = Microsoft Authenticator, with YubiKey as fallback.</t>
   </si>
   <si>
     <t xml:space="preserve">Baseline Security &gt; Multi-Factor Authentication; new "Authentication Methods" subsection</t>
@@ -736,6 +702,9 @@
 Who is authorised to sign the porting LOA, and does the billing name and service address match the carrier record exactly?
 Which users get a DID versus Teams calling with no number — do shop-floor users need phones at all?
 Which auto attendants, call queues, hunt groups, after-hours routing, and reception/overflow behaviours are in use today and must be rebuilt (each needs a resource account and service number)?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Licensing plan implies phone service for the 55 BP-tier users (Teams Phone Standard) plus the 15 G5 users (included in G5); the 80 frontline users get no phone service.</t>
   </si>
   <si>
     <t xml:space="preserve">Teams Voice &gt; Numbering and Number Porting; Voice Features</t>
@@ -1070,6 +1039,30 @@
   </si>
   <si>
     <t xml:space="preserve">Config action: disable Entra Connect against the commercial tenant at cutover; WMP decommissions the old tenant fully thereafter.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">G-07</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Entra ID P2 purchase vehicle</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Settled by the licensing plan: P2 arrives via M365 G5 (15 users) and the F5 Security + Compliance add-on (80 users); the 55-seat BP + Defender/Purview Suite tier's P2 entitlement is verified under G-06.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">No separate purchase decision remains. Entra P2 coverage verification for the 55-seat tier is tracked in G-06.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">G-09</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Device join model (design/WBS contradiction)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Pure Entra join.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Design/config actions: end state is Entra ID join (cloud-only). Simplify CA policy 3's grant to require-compliant-device only; remove the Seamless SSO section (a domain-joined-only feature); both join states coexist only during migration waves. Supersedes WBS 1.3.2's hybrid-join note. Cascade: closes G-08's sign-in-method question (PHS alone).</t>
   </si>
   <si>
     <t xml:space="preserve">G-10</t>
@@ -1988,7 +1981,7 @@
       </c>
       <c r="F21" s="9" t="n">
         <f aca="false">COUNTIF('Gap Register'!J:J,"High")</f>
-        <v>29</v>
+        <v>27</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2013,7 +2006,7 @@
       </c>
       <c r="C23" s="9" t="n">
         <f aca="false">COUNTIF('Gap Register'!B:B,B23)</f>
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E23" s="8" t="s">
         <v>20</v>
@@ -2029,14 +2022,14 @@
       </c>
       <c r="C24" s="9" t="n">
         <f aca="false">COUNTIF('Gap Register'!B:B,B24)</f>
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E24" s="10" t="s">
         <v>22</v>
       </c>
       <c r="F24" s="11" t="n">
         <f aca="false">COUNTA('Gap Register'!A:A)-1</f>
-        <v>43</v>
+        <v>41</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2052,7 +2045,7 @@
       </c>
       <c r="F25" s="11" t="n">
         <f aca="false">COUNTA('Resolved Decisions'!A:A)-1</f>
-        <v>21</v>
+        <v>23</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2149,7 +2142,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:K44"/>
+  <dimension ref="A1:K42"/>
   <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="7"/>
@@ -2338,7 +2331,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="6" customFormat="false" ht="68.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="6" customFormat="false" ht="113.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="13" t="s">
         <v>72</v>
       </c>
@@ -2373,18 +2366,18 @@
         <v>50</v>
       </c>
     </row>
-    <row r="7" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="7" customFormat="false" ht="91" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="13" t="s">
         <v>79</v>
       </c>
       <c r="B7" s="13" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="C7" s="13" t="s">
         <v>80</v>
       </c>
       <c r="D7" s="13" t="s">
-        <v>67</v>
+        <v>74</v>
       </c>
       <c r="E7" s="13" t="s">
         <v>81</v>
@@ -2399,16 +2392,16 @@
         <v>84</v>
       </c>
       <c r="I7" s="13" t="s">
-        <v>57</v>
-      </c>
-      <c r="J7" s="15" t="s">
-        <v>64</v>
+        <v>48</v>
+      </c>
+      <c r="J7" s="14" t="s">
+        <v>49</v>
       </c>
       <c r="K7" s="13" t="s">
         <v>50</v>
       </c>
     </row>
-    <row r="8" customFormat="false" ht="113.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="8" customFormat="false" ht="68.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="13" t="s">
         <v>85</v>
       </c>
@@ -2434,16 +2427,16 @@
         <v>90</v>
       </c>
       <c r="I8" s="13" t="s">
-        <v>48</v>
-      </c>
-      <c r="J8" s="14" t="s">
-        <v>49</v>
+        <v>57</v>
+      </c>
+      <c r="J8" s="15" t="s">
+        <v>64</v>
       </c>
       <c r="K8" s="13" t="s">
         <v>50</v>
       </c>
     </row>
-    <row r="9" customFormat="false" ht="91" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="9" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="13" t="s">
         <v>91</v>
       </c>
@@ -2469,16 +2462,16 @@
         <v>96</v>
       </c>
       <c r="I9" s="13" t="s">
-        <v>48</v>
-      </c>
-      <c r="J9" s="14" t="s">
-        <v>49</v>
+        <v>57</v>
+      </c>
+      <c r="J9" s="15" t="s">
+        <v>64</v>
       </c>
       <c r="K9" s="13" t="s">
         <v>50</v>
       </c>
     </row>
-    <row r="10" customFormat="false" ht="79.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="10" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="13" t="s">
         <v>97</v>
       </c>
@@ -2489,7 +2482,7 @@
         <v>98</v>
       </c>
       <c r="D10" s="13" t="s">
-        <v>74</v>
+        <v>53</v>
       </c>
       <c r="E10" s="13" t="s">
         <v>99</v>
@@ -2506,8 +2499,8 @@
       <c r="I10" s="13" t="s">
         <v>57</v>
       </c>
-      <c r="J10" s="14" t="s">
-        <v>49</v>
+      <c r="J10" s="15" t="s">
+        <v>64</v>
       </c>
       <c r="K10" s="13" t="s">
         <v>50</v>
@@ -2518,7 +2511,7 @@
         <v>103</v>
       </c>
       <c r="B11" s="13" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="C11" s="13" t="s">
         <v>104</v>
@@ -2539,7 +2532,7 @@
         <v>108</v>
       </c>
       <c r="I11" s="13" t="s">
-        <v>57</v>
+        <v>48</v>
       </c>
       <c r="J11" s="15" t="s">
         <v>64</v>
@@ -2553,7 +2546,7 @@
         <v>109</v>
       </c>
       <c r="B12" s="13" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="C12" s="13" t="s">
         <v>110</v>
@@ -2574,42 +2567,42 @@
         <v>114</v>
       </c>
       <c r="I12" s="13" t="s">
-        <v>57</v>
-      </c>
-      <c r="J12" s="15" t="s">
-        <v>64</v>
+        <v>115</v>
+      </c>
+      <c r="J12" s="14" t="s">
+        <v>49</v>
       </c>
       <c r="K12" s="13" t="s">
         <v>50</v>
       </c>
     </row>
-    <row r="13" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="13" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="13" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="B13" s="13" t="s">
         <v>23</v>
       </c>
       <c r="C13" s="13" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="D13" s="13" t="s">
         <v>74</v>
       </c>
       <c r="E13" s="13" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="F13" s="13" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="G13" s="13" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="H13" s="13" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="I13" s="13" t="s">
-        <v>48</v>
+        <v>57</v>
       </c>
       <c r="J13" s="15" t="s">
         <v>64</v>
@@ -2618,33 +2611,31 @@
         <v>50</v>
       </c>
     </row>
-    <row r="14" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="14" customFormat="false" ht="124.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="13" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="B14" s="13" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="C14" s="13" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="D14" s="13" t="s">
-        <v>53</v>
+        <v>67</v>
       </c>
       <c r="E14" s="13" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="F14" s="13" t="s">
-        <v>124</v>
-      </c>
-      <c r="G14" s="13" t="s">
         <v>125</v>
       </c>
+      <c r="G14" s="13"/>
       <c r="H14" s="13" t="s">
         <v>126</v>
       </c>
       <c r="I14" s="13" t="s">
-        <v>127</v>
+        <v>57</v>
       </c>
       <c r="J14" s="14" t="s">
         <v>49</v>
@@ -2653,33 +2644,33 @@
         <v>50</v>
       </c>
     </row>
-    <row r="15" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="15" customFormat="false" ht="68.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="13" t="s">
+        <v>127</v>
+      </c>
+      <c r="B15" s="13" t="s">
+        <v>25</v>
+      </c>
+      <c r="C15" s="13" t="s">
         <v>128</v>
-      </c>
-      <c r="B15" s="13" t="s">
-        <v>23</v>
-      </c>
-      <c r="C15" s="13" t="s">
-        <v>129</v>
       </c>
       <c r="D15" s="13" t="s">
         <v>74</v>
       </c>
       <c r="E15" s="13" t="s">
+        <v>129</v>
+      </c>
+      <c r="F15" s="13" t="s">
         <v>130</v>
       </c>
-      <c r="F15" s="13" t="s">
+      <c r="G15" s="13" t="s">
         <v>131</v>
       </c>
-      <c r="G15" s="13" t="s">
+      <c r="H15" s="13" t="s">
         <v>132</v>
       </c>
-      <c r="H15" s="13" t="s">
-        <v>133</v>
-      </c>
       <c r="I15" s="13" t="s">
-        <v>57</v>
+        <v>48</v>
       </c>
       <c r="J15" s="15" t="s">
         <v>64</v>
@@ -2688,45 +2679,47 @@
         <v>50</v>
       </c>
     </row>
-    <row r="16" customFormat="false" ht="124.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="16" customFormat="false" ht="91" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="13" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="B16" s="13" t="s">
         <v>25</v>
       </c>
       <c r="C16" s="13" t="s">
+        <v>134</v>
+      </c>
+      <c r="D16" s="13" t="s">
+        <v>53</v>
+      </c>
+      <c r="E16" s="13" t="s">
         <v>135</v>
       </c>
-      <c r="D16" s="13" t="s">
-        <v>67</v>
-      </c>
-      <c r="E16" s="13" t="s">
+      <c r="F16" s="13" t="s">
         <v>136</v>
       </c>
-      <c r="F16" s="13" t="s">
+      <c r="G16" s="13" t="s">
         <v>137</v>
       </c>
-      <c r="G16" s="13"/>
       <c r="H16" s="13" t="s">
         <v>138</v>
       </c>
       <c r="I16" s="13" t="s">
         <v>57</v>
       </c>
-      <c r="J16" s="14" t="s">
-        <v>49</v>
+      <c r="J16" s="15" t="s">
+        <v>64</v>
       </c>
       <c r="K16" s="13" t="s">
         <v>50</v>
       </c>
     </row>
-    <row r="17" customFormat="false" ht="68.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="17" customFormat="false" ht="102.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="13" t="s">
         <v>139</v>
       </c>
       <c r="B17" s="13" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="C17" s="13" t="s">
         <v>140</v>
@@ -2740,17 +2733,15 @@
       <c r="F17" s="13" t="s">
         <v>142</v>
       </c>
-      <c r="G17" s="13" t="s">
+      <c r="G17" s="13"/>
+      <c r="H17" s="13" t="s">
         <v>143</v>
       </c>
-      <c r="H17" s="13" t="s">
-        <v>144</v>
-      </c>
       <c r="I17" s="13" t="s">
-        <v>48</v>
-      </c>
-      <c r="J17" s="15" t="s">
-        <v>64</v>
+        <v>57</v>
+      </c>
+      <c r="J17" s="14" t="s">
+        <v>49</v>
       </c>
       <c r="K17" s="13" t="s">
         <v>50</v>
@@ -2758,67 +2749,69 @@
     </row>
     <row r="18" customFormat="false" ht="91" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="13" t="s">
+        <v>144</v>
+      </c>
+      <c r="B18" s="13" t="s">
+        <v>26</v>
+      </c>
+      <c r="C18" s="13" t="s">
         <v>145</v>
-      </c>
-      <c r="B18" s="13" t="s">
-        <v>25</v>
-      </c>
-      <c r="C18" s="13" t="s">
-        <v>146</v>
       </c>
       <c r="D18" s="13" t="s">
         <v>53</v>
       </c>
       <c r="E18" s="13" t="s">
+        <v>146</v>
+      </c>
+      <c r="F18" s="13" t="s">
         <v>147</v>
       </c>
-      <c r="F18" s="13" t="s">
+      <c r="G18" s="13" t="s">
         <v>148</v>
       </c>
-      <c r="G18" s="13" t="s">
+      <c r="H18" s="13" t="s">
         <v>149</v>
-      </c>
-      <c r="H18" s="13" t="s">
-        <v>150</v>
       </c>
       <c r="I18" s="13" t="s">
         <v>57</v>
       </c>
-      <c r="J18" s="15" t="s">
-        <v>64</v>
+      <c r="J18" s="14" t="s">
+        <v>49</v>
       </c>
       <c r="K18" s="13" t="s">
         <v>50</v>
       </c>
     </row>
-    <row r="19" customFormat="false" ht="102.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="19" customFormat="false" ht="68.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="13" t="s">
+        <v>150</v>
+      </c>
+      <c r="B19" s="13" t="s">
+        <v>15</v>
+      </c>
+      <c r="C19" s="13" t="s">
         <v>151</v>
-      </c>
-      <c r="B19" s="13" t="s">
-        <v>26</v>
-      </c>
-      <c r="C19" s="13" t="s">
-        <v>152</v>
       </c>
       <c r="D19" s="13" t="s">
         <v>74</v>
       </c>
       <c r="E19" s="13" t="s">
+        <v>152</v>
+      </c>
+      <c r="F19" s="13" t="s">
         <v>153</v>
       </c>
-      <c r="F19" s="13" t="s">
+      <c r="G19" s="13" t="s">
         <v>154</v>
       </c>
-      <c r="G19" s="13"/>
       <c r="H19" s="13" t="s">
-        <v>155</v>
+        <v>47</v>
       </c>
       <c r="I19" s="13" t="s">
-        <v>57</v>
-      </c>
-      <c r="J19" s="14" t="s">
-        <v>49</v>
+        <v>48</v>
+      </c>
+      <c r="J19" s="15" t="s">
+        <v>64</v>
       </c>
       <c r="K19" s="13" t="s">
         <v>50</v>
@@ -2826,31 +2819,31 @@
     </row>
     <row r="20" customFormat="false" ht="91" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="13" t="s">
+        <v>155</v>
+      </c>
+      <c r="B20" s="13" t="s">
+        <v>15</v>
+      </c>
+      <c r="C20" s="13" t="s">
         <v>156</v>
       </c>
-      <c r="B20" s="13" t="s">
-        <v>26</v>
-      </c>
-      <c r="C20" s="13" t="s">
+      <c r="D20" s="13" t="s">
+        <v>74</v>
+      </c>
+      <c r="E20" s="13" t="s">
         <v>157</v>
       </c>
-      <c r="D20" s="13" t="s">
-        <v>53</v>
-      </c>
-      <c r="E20" s="13" t="s">
+      <c r="F20" s="13" t="s">
         <v>158</v>
       </c>
-      <c r="F20" s="13" t="s">
+      <c r="G20" s="13" t="s">
         <v>159</v>
       </c>
-      <c r="G20" s="13" t="s">
+      <c r="H20" s="13" t="s">
         <v>160</v>
       </c>
-      <c r="H20" s="13" t="s">
-        <v>161</v>
-      </c>
       <c r="I20" s="13" t="s">
-        <v>57</v>
+        <v>48</v>
       </c>
       <c r="J20" s="14" t="s">
         <v>49</v>
@@ -2859,42 +2852,42 @@
         <v>50</v>
       </c>
     </row>
-    <row r="21" customFormat="false" ht="68.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="21" customFormat="false" ht="102.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="13" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="B21" s="13" t="s">
         <v>15</v>
       </c>
       <c r="C21" s="13" t="s">
+        <v>162</v>
+      </c>
+      <c r="D21" s="13" t="s">
+        <v>53</v>
+      </c>
+      <c r="E21" s="13" t="s">
         <v>163</v>
       </c>
-      <c r="D21" s="13" t="s">
-        <v>74</v>
-      </c>
-      <c r="E21" s="13" t="s">
+      <c r="F21" s="13" t="s">
         <v>164</v>
       </c>
-      <c r="F21" s="13" t="s">
+      <c r="G21" s="13" t="s">
         <v>165</v>
       </c>
-      <c r="G21" s="13" t="s">
+      <c r="H21" s="13" t="s">
         <v>166</v>
       </c>
-      <c r="H21" s="13" t="s">
-        <v>47</v>
-      </c>
       <c r="I21" s="13" t="s">
-        <v>48</v>
-      </c>
-      <c r="J21" s="15" t="s">
-        <v>64</v>
+        <v>57</v>
+      </c>
+      <c r="J21" s="14" t="s">
+        <v>49</v>
       </c>
       <c r="K21" s="13" t="s">
         <v>50</v>
       </c>
     </row>
-    <row r="22" customFormat="false" ht="91" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="22" customFormat="false" ht="102.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="13" t="s">
         <v>167</v>
       </c>
@@ -2913,14 +2906,12 @@
       <c r="F22" s="13" t="s">
         <v>170</v>
       </c>
-      <c r="G22" s="13" t="s">
+      <c r="G22" s="13"/>
+      <c r="H22" s="13" t="s">
         <v>171</v>
       </c>
-      <c r="H22" s="13" t="s">
-        <v>172</v>
-      </c>
       <c r="I22" s="13" t="s">
-        <v>48</v>
+        <v>57</v>
       </c>
       <c r="J22" s="14" t="s">
         <v>49</v>
@@ -2929,30 +2920,28 @@
         <v>50</v>
       </c>
     </row>
-    <row r="23" customFormat="false" ht="102.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="23" customFormat="false" ht="91" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="13" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="B23" s="13" t="s">
         <v>15</v>
       </c>
       <c r="C23" s="13" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="D23" s="13" t="s">
         <v>53</v>
       </c>
       <c r="E23" s="13" t="s">
+        <v>174</v>
+      </c>
+      <c r="F23" s="13" t="s">
         <v>175</v>
       </c>
-      <c r="F23" s="13" t="s">
+      <c r="G23" s="13"/>
+      <c r="H23" s="13" t="s">
         <v>176</v>
-      </c>
-      <c r="G23" s="13" t="s">
-        <v>177</v>
-      </c>
-      <c r="H23" s="13" t="s">
-        <v>178</v>
       </c>
       <c r="I23" s="13" t="s">
         <v>57</v>
@@ -2964,97 +2953,99 @@
         <v>50</v>
       </c>
     </row>
-    <row r="24" customFormat="false" ht="102.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="24" customFormat="false" ht="68.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="13" t="s">
-        <v>179</v>
+        <v>177</v>
       </c>
       <c r="B24" s="13" t="s">
         <v>15</v>
       </c>
       <c r="C24" s="13" t="s">
+        <v>178</v>
+      </c>
+      <c r="D24" s="13" t="s">
+        <v>53</v>
+      </c>
+      <c r="E24" s="13" t="s">
+        <v>179</v>
+      </c>
+      <c r="F24" s="13" t="s">
         <v>180</v>
-      </c>
-      <c r="D24" s="13" t="s">
-        <v>74</v>
-      </c>
-      <c r="E24" s="13" t="s">
-        <v>181</v>
-      </c>
-      <c r="F24" s="13" t="s">
-        <v>182</v>
       </c>
       <c r="G24" s="13"/>
       <c r="H24" s="13" t="s">
-        <v>183</v>
+        <v>181</v>
       </c>
       <c r="I24" s="13" t="s">
-        <v>57</v>
-      </c>
-      <c r="J24" s="14" t="s">
-        <v>49</v>
+        <v>115</v>
+      </c>
+      <c r="J24" s="15" t="s">
+        <v>64</v>
       </c>
       <c r="K24" s="13" t="s">
         <v>50</v>
       </c>
     </row>
-    <row r="25" customFormat="false" ht="91" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="25" customFormat="false" ht="113.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="13" t="s">
-        <v>184</v>
+        <v>182</v>
       </c>
       <c r="B25" s="13" t="s">
         <v>15</v>
       </c>
       <c r="C25" s="13" t="s">
+        <v>183</v>
+      </c>
+      <c r="D25" s="13" t="s">
+        <v>67</v>
+      </c>
+      <c r="E25" s="13" t="s">
+        <v>184</v>
+      </c>
+      <c r="F25" s="13" t="s">
         <v>185</v>
-      </c>
-      <c r="D25" s="13" t="s">
-        <v>53</v>
-      </c>
-      <c r="E25" s="13" t="s">
-        <v>186</v>
-      </c>
-      <c r="F25" s="13" t="s">
-        <v>187</v>
       </c>
       <c r="G25" s="13"/>
       <c r="H25" s="13" t="s">
-        <v>188</v>
+        <v>186</v>
       </c>
       <c r="I25" s="13" t="s">
         <v>57</v>
       </c>
-      <c r="J25" s="14" t="s">
-        <v>49</v>
+      <c r="J25" s="15" t="s">
+        <v>64</v>
       </c>
       <c r="K25" s="13" t="s">
         <v>50</v>
       </c>
     </row>
-    <row r="26" customFormat="false" ht="68.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="26" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="13" t="s">
+        <v>187</v>
+      </c>
+      <c r="B26" s="13" t="s">
+        <v>27</v>
+      </c>
+      <c r="C26" s="13" t="s">
+        <v>188</v>
+      </c>
+      <c r="D26" s="13" t="s">
+        <v>67</v>
+      </c>
+      <c r="E26" s="13" t="s">
         <v>189</v>
       </c>
-      <c r="B26" s="13" t="s">
-        <v>15</v>
-      </c>
-      <c r="C26" s="13" t="s">
+      <c r="F26" s="13" t="s">
         <v>190</v>
       </c>
-      <c r="D26" s="13" t="s">
-        <v>53</v>
-      </c>
-      <c r="E26" s="13" t="s">
+      <c r="G26" s="13" t="s">
         <v>191</v>
       </c>
-      <c r="F26" s="13" t="s">
+      <c r="H26" s="13" t="s">
         <v>192</v>
       </c>
-      <c r="G26" s="13"/>
-      <c r="H26" s="13" t="s">
+      <c r="I26" s="13" t="s">
         <v>193</v>
-      </c>
-      <c r="I26" s="13" t="s">
-        <v>127</v>
       </c>
       <c r="J26" s="15" t="s">
         <v>64</v>
@@ -3063,18 +3054,18 @@
         <v>50</v>
       </c>
     </row>
-    <row r="27" customFormat="false" ht="113.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="27" customFormat="false" ht="124.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="13" t="s">
         <v>194</v>
       </c>
       <c r="B27" s="13" t="s">
-        <v>15</v>
+        <v>27</v>
       </c>
       <c r="C27" s="13" t="s">
         <v>195</v>
       </c>
       <c r="D27" s="13" t="s">
-        <v>67</v>
+        <v>53</v>
       </c>
       <c r="E27" s="13" t="s">
         <v>196</v>
@@ -3082,56 +3073,56 @@
       <c r="F27" s="13" t="s">
         <v>197</v>
       </c>
-      <c r="G27" s="13"/>
+      <c r="G27" s="13" t="s">
+        <v>198</v>
+      </c>
       <c r="H27" s="13" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="I27" s="13" t="s">
-        <v>57</v>
-      </c>
-      <c r="J27" s="15" t="s">
-        <v>64</v>
+        <v>200</v>
+      </c>
+      <c r="J27" s="14" t="s">
+        <v>49</v>
       </c>
       <c r="K27" s="13" t="s">
         <v>50</v>
       </c>
     </row>
-    <row r="28" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="28" customFormat="false" ht="102.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="13" t="s">
-        <v>199</v>
+        <v>201</v>
       </c>
       <c r="B28" s="13" t="s">
         <v>27</v>
       </c>
       <c r="C28" s="13" t="s">
+        <v>202</v>
+      </c>
+      <c r="D28" s="13" t="s">
+        <v>53</v>
+      </c>
+      <c r="E28" s="13" t="s">
+        <v>203</v>
+      </c>
+      <c r="F28" s="13" t="s">
+        <v>204</v>
+      </c>
+      <c r="G28" s="13"/>
+      <c r="H28" s="13" t="s">
+        <v>205</v>
+      </c>
+      <c r="I28" s="13" t="s">
         <v>200</v>
       </c>
-      <c r="D28" s="13" t="s">
-        <v>67</v>
-      </c>
-      <c r="E28" s="13" t="s">
-        <v>201</v>
-      </c>
-      <c r="F28" s="13" t="s">
-        <v>202</v>
-      </c>
-      <c r="G28" s="13" t="s">
-        <v>203</v>
-      </c>
-      <c r="H28" s="13" t="s">
-        <v>204</v>
-      </c>
-      <c r="I28" s="13" t="s">
-        <v>205</v>
-      </c>
-      <c r="J28" s="15" t="s">
-        <v>64</v>
+      <c r="J28" s="14" t="s">
+        <v>49</v>
       </c>
       <c r="K28" s="13" t="s">
         <v>50</v>
       </c>
     </row>
-    <row r="29" customFormat="false" ht="124.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="29" customFormat="false" ht="102.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="13" t="s">
         <v>206</v>
       </c>
@@ -3155,7 +3146,7 @@
         <v>210</v>
       </c>
       <c r="I29" s="13" t="s">
-        <v>211</v>
+        <v>200</v>
       </c>
       <c r="J29" s="14" t="s">
         <v>49</v>
@@ -3164,31 +3155,33 @@
         <v>50</v>
       </c>
     </row>
-    <row r="30" customFormat="false" ht="102.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="30" customFormat="false" ht="113.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="13" t="s">
+        <v>211</v>
+      </c>
+      <c r="B30" s="13" t="s">
+        <v>28</v>
+      </c>
+      <c r="C30" s="13" t="s">
         <v>212</v>
-      </c>
-      <c r="B30" s="13" t="s">
-        <v>27</v>
-      </c>
-      <c r="C30" s="13" t="s">
-        <v>213</v>
       </c>
       <c r="D30" s="13" t="s">
         <v>53</v>
       </c>
       <c r="E30" s="13" t="s">
+        <v>213</v>
+      </c>
+      <c r="F30" s="13" t="s">
         <v>214</v>
       </c>
-      <c r="F30" s="13" t="s">
+      <c r="G30" s="13" t="s">
         <v>215</v>
       </c>
-      <c r="G30" s="13"/>
       <c r="H30" s="13" t="s">
         <v>216</v>
       </c>
       <c r="I30" s="13" t="s">
-        <v>211</v>
+        <v>57</v>
       </c>
       <c r="J30" s="14" t="s">
         <v>49</v>
@@ -3197,18 +3190,18 @@
         <v>50</v>
       </c>
     </row>
-    <row r="31" customFormat="false" ht="102.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="31" customFormat="false" ht="79.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="13" t="s">
         <v>217</v>
       </c>
       <c r="B31" s="13" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="C31" s="13" t="s">
         <v>218</v>
       </c>
       <c r="D31" s="13" t="s">
-        <v>53</v>
+        <v>74</v>
       </c>
       <c r="E31" s="13" t="s">
         <v>219</v>
@@ -3216,12 +3209,14 @@
       <c r="F31" s="13" t="s">
         <v>220</v>
       </c>
-      <c r="G31" s="13"/>
+      <c r="G31" s="13" t="s">
+        <v>221</v>
+      </c>
       <c r="H31" s="13" t="s">
-        <v>221</v>
+        <v>222</v>
       </c>
       <c r="I31" s="13" t="s">
-        <v>211</v>
+        <v>57</v>
       </c>
       <c r="J31" s="14" t="s">
         <v>49</v>
@@ -3230,28 +3225,26 @@
         <v>50</v>
       </c>
     </row>
-    <row r="32" customFormat="false" ht="113.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="32" customFormat="false" ht="79.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="13" t="s">
-        <v>222</v>
+        <v>223</v>
       </c>
       <c r="B32" s="13" t="s">
         <v>28</v>
       </c>
       <c r="C32" s="13" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
       <c r="D32" s="13" t="s">
         <v>53</v>
       </c>
       <c r="E32" s="13" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="F32" s="13" t="s">
-        <v>225</v>
-      </c>
-      <c r="G32" s="13" t="s">
         <v>226</v>
       </c>
+      <c r="G32" s="13"/>
       <c r="H32" s="13" t="s">
         <v>227</v>
       </c>
@@ -3265,7 +3258,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="33" customFormat="false" ht="79.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="33" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="13" t="s">
         <v>228</v>
       </c>
@@ -3293,8 +3286,8 @@
       <c r="I33" s="13" t="s">
         <v>57</v>
       </c>
-      <c r="J33" s="14" t="s">
-        <v>49</v>
+      <c r="J33" s="15" t="s">
+        <v>64</v>
       </c>
       <c r="K33" s="13" t="s">
         <v>50</v>
@@ -3305,7 +3298,7 @@
         <v>234</v>
       </c>
       <c r="B34" s="13" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="C34" s="13" t="s">
         <v>235</v>
@@ -3319,12 +3312,14 @@
       <c r="F34" s="13" t="s">
         <v>237</v>
       </c>
-      <c r="G34" s="13"/>
+      <c r="G34" s="13" t="s">
+        <v>238</v>
+      </c>
       <c r="H34" s="13" t="s">
-        <v>238</v>
+        <v>239</v>
       </c>
       <c r="I34" s="13" t="s">
-        <v>57</v>
+        <v>115</v>
       </c>
       <c r="J34" s="14" t="s">
         <v>49</v>
@@ -3333,42 +3328,40 @@
         <v>50</v>
       </c>
     </row>
-    <row r="35" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="35" customFormat="false" ht="124.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="13" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
       <c r="B35" s="13" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="C35" s="13" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="D35" s="13" t="s">
         <v>74</v>
       </c>
       <c r="E35" s="13" t="s">
-        <v>241</v>
+        <v>242</v>
       </c>
       <c r="F35" s="13" t="s">
-        <v>242</v>
-      </c>
-      <c r="G35" s="13" t="s">
         <v>243</v>
       </c>
+      <c r="G35" s="13"/>
       <c r="H35" s="13" t="s">
         <v>244</v>
       </c>
       <c r="I35" s="13" t="s">
-        <v>57</v>
-      </c>
-      <c r="J35" s="15" t="s">
-        <v>64</v>
+        <v>48</v>
+      </c>
+      <c r="J35" s="14" t="s">
+        <v>49</v>
       </c>
       <c r="K35" s="13" t="s">
         <v>50</v>
       </c>
     </row>
-    <row r="36" customFormat="false" ht="79.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="36" customFormat="false" ht="102.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="13" t="s">
         <v>245</v>
       </c>
@@ -3379,7 +3372,7 @@
         <v>246</v>
       </c>
       <c r="D36" s="13" t="s">
-        <v>53</v>
+        <v>74</v>
       </c>
       <c r="E36" s="13" t="s">
         <v>247</v>
@@ -3394,7 +3387,7 @@
         <v>250</v>
       </c>
       <c r="I36" s="13" t="s">
-        <v>127</v>
+        <v>57</v>
       </c>
       <c r="J36" s="14" t="s">
         <v>49</v>
@@ -3403,12 +3396,12 @@
         <v>50</v>
       </c>
     </row>
-    <row r="37" customFormat="false" ht="124.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="37" customFormat="false" ht="79.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="13" t="s">
         <v>251</v>
       </c>
       <c r="B37" s="13" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="C37" s="13" t="s">
         <v>252</v>
@@ -3427,7 +3420,7 @@
         <v>255</v>
       </c>
       <c r="I37" s="13" t="s">
-        <v>48</v>
+        <v>57</v>
       </c>
       <c r="J37" s="14" t="s">
         <v>49</v>
@@ -3441,7 +3434,7 @@
         <v>256</v>
       </c>
       <c r="B38" s="13" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="C38" s="13" t="s">
         <v>257</v>
@@ -3455,42 +3448,42 @@
       <c r="F38" s="13" t="s">
         <v>259</v>
       </c>
-      <c r="G38" s="13" t="s">
+      <c r="G38" s="13"/>
+      <c r="H38" s="13" t="s">
         <v>260</v>
-      </c>
-      <c r="H38" s="13" t="s">
-        <v>261</v>
       </c>
       <c r="I38" s="13" t="s">
         <v>57</v>
       </c>
-      <c r="J38" s="14" t="s">
-        <v>49</v>
+      <c r="J38" s="15" t="s">
+        <v>64</v>
       </c>
       <c r="K38" s="13" t="s">
         <v>50</v>
       </c>
     </row>
-    <row r="39" customFormat="false" ht="79.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="39" customFormat="false" ht="91" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="13" t="s">
+        <v>261</v>
+      </c>
+      <c r="B39" s="13" t="s">
+        <v>31</v>
+      </c>
+      <c r="C39" s="13" t="s">
         <v>262</v>
       </c>
-      <c r="B39" s="13" t="s">
-        <v>30</v>
-      </c>
-      <c r="C39" s="13" t="s">
+      <c r="D39" s="13" t="s">
+        <v>67</v>
+      </c>
+      <c r="E39" s="13" t="s">
         <v>263</v>
       </c>
-      <c r="D39" s="13" t="s">
-        <v>74</v>
-      </c>
-      <c r="E39" s="13" t="s">
+      <c r="F39" s="13" t="s">
         <v>264</v>
       </c>
-      <c r="F39" s="13" t="s">
+      <c r="G39" s="13" t="s">
         <v>265</v>
       </c>
-      <c r="G39" s="13"/>
       <c r="H39" s="13" t="s">
         <v>266</v>
       </c>
@@ -3504,12 +3497,12 @@
         <v>50</v>
       </c>
     </row>
-    <row r="40" customFormat="false" ht="102.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="40" customFormat="false" ht="91" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="13" t="s">
         <v>267</v>
       </c>
       <c r="B40" s="13" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="C40" s="13" t="s">
         <v>268</v>
@@ -3523,44 +3516,46 @@
       <c r="F40" s="13" t="s">
         <v>270</v>
       </c>
-      <c r="G40" s="13"/>
+      <c r="G40" s="13" t="s">
+        <v>271</v>
+      </c>
       <c r="H40" s="13" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
       <c r="I40" s="13" t="s">
         <v>57</v>
       </c>
-      <c r="J40" s="15" t="s">
-        <v>64</v>
+      <c r="J40" s="14" t="s">
+        <v>49</v>
       </c>
       <c r="K40" s="13" t="s">
         <v>50</v>
       </c>
     </row>
-    <row r="41" customFormat="false" ht="91" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="41" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="13" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="B41" s="13" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="C41" s="13" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="D41" s="13" t="s">
-        <v>67</v>
+        <v>74</v>
       </c>
       <c r="E41" s="13" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
       <c r="F41" s="13" t="s">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="G41" s="13" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
       <c r="H41" s="13" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
       <c r="I41" s="13" t="s">
         <v>57</v>
@@ -3572,33 +3567,33 @@
         <v>50</v>
       </c>
     </row>
-    <row r="42" customFormat="false" ht="91" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="42" customFormat="false" ht="102.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="13" t="s">
-        <v>278</v>
+        <v>279</v>
       </c>
       <c r="B42" s="13" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="C42" s="13" t="s">
-        <v>279</v>
+        <v>280</v>
       </c>
       <c r="D42" s="13" t="s">
         <v>74</v>
       </c>
       <c r="E42" s="13" t="s">
-        <v>280</v>
+        <v>281</v>
       </c>
       <c r="F42" s="13" t="s">
-        <v>281</v>
+        <v>282</v>
       </c>
       <c r="G42" s="13" t="s">
-        <v>282</v>
+        <v>283</v>
       </c>
       <c r="H42" s="13" t="s">
-        <v>283</v>
+        <v>284</v>
       </c>
       <c r="I42" s="13" t="s">
-        <v>57</v>
+        <v>285</v>
       </c>
       <c r="J42" s="14" t="s">
         <v>49</v>
@@ -3607,78 +3602,8 @@
         <v>50</v>
       </c>
     </row>
-    <row r="43" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A43" s="13" t="s">
-        <v>284</v>
-      </c>
-      <c r="B43" s="13" t="s">
-        <v>32</v>
-      </c>
-      <c r="C43" s="13" t="s">
-        <v>285</v>
-      </c>
-      <c r="D43" s="13" t="s">
-        <v>74</v>
-      </c>
-      <c r="E43" s="13" t="s">
-        <v>286</v>
-      </c>
-      <c r="F43" s="13" t="s">
-        <v>287</v>
-      </c>
-      <c r="G43" s="13" t="s">
-        <v>288</v>
-      </c>
-      <c r="H43" s="13" t="s">
-        <v>289</v>
-      </c>
-      <c r="I43" s="13" t="s">
-        <v>57</v>
-      </c>
-      <c r="J43" s="14" t="s">
-        <v>49</v>
-      </c>
-      <c r="K43" s="13" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="44" customFormat="false" ht="102.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A44" s="13" t="s">
-        <v>290</v>
-      </c>
-      <c r="B44" s="13" t="s">
-        <v>32</v>
-      </c>
-      <c r="C44" s="13" t="s">
-        <v>291</v>
-      </c>
-      <c r="D44" s="13" t="s">
-        <v>74</v>
-      </c>
-      <c r="E44" s="13" t="s">
-        <v>292</v>
-      </c>
-      <c r="F44" s="13" t="s">
-        <v>293</v>
-      </c>
-      <c r="G44" s="13" t="s">
-        <v>294</v>
-      </c>
-      <c r="H44" s="13" t="s">
-        <v>295</v>
-      </c>
-      <c r="I44" s="13" t="s">
-        <v>296</v>
-      </c>
-      <c r="J44" s="14" t="s">
-        <v>49</v>
-      </c>
-      <c r="K44" s="13" t="s">
-        <v>50</v>
-      </c>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:K44"/>
+  <autoFilter ref="A1:K42"/>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
@@ -3695,7 +3620,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:E22"/>
+  <dimension ref="A1:E24"/>
   <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="7"/>
@@ -3712,374 +3637,408 @@
         <v>34</v>
       </c>
       <c r="C1" s="12" t="s">
-        <v>297</v>
+        <v>286</v>
       </c>
       <c r="D1" s="12" t="s">
-        <v>298</v>
+        <v>287</v>
       </c>
       <c r="E1" s="12" t="s">
-        <v>299</v>
+        <v>288</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="13" t="s">
-        <v>300</v>
+        <v>289</v>
       </c>
       <c r="B2" s="13" t="s">
         <v>17</v>
       </c>
       <c r="C2" s="13" t="s">
+        <v>290</v>
+      </c>
+      <c r="D2" s="13" t="s">
+        <v>291</v>
+      </c>
+      <c r="E2" s="13" t="s">
+        <v>292</v>
+      </c>
+    </row>
+    <row r="3" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A3" s="13" t="s">
+        <v>293</v>
+      </c>
+      <c r="B3" s="13" t="s">
+        <v>19</v>
+      </c>
+      <c r="C3" s="13" t="s">
+        <v>294</v>
+      </c>
+      <c r="D3" s="13" t="s">
+        <v>295</v>
+      </c>
+      <c r="E3" s="13" t="s">
+        <v>296</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="13" t="s">
+        <v>297</v>
+      </c>
+      <c r="B4" s="13" t="s">
+        <v>21</v>
+      </c>
+      <c r="C4" s="13" t="s">
+        <v>298</v>
+      </c>
+      <c r="D4" s="13" t="s">
+        <v>299</v>
+      </c>
+      <c r="E4" s="13" t="s">
+        <v>300</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="13" t="s">
         <v>301</v>
       </c>
-      <c r="D2" s="13" t="s">
+      <c r="B5" s="13" t="s">
+        <v>21</v>
+      </c>
+      <c r="C5" s="13" t="s">
         <v>302</v>
       </c>
-      <c r="E2" s="13" t="s">
+      <c r="D5" s="13" t="s">
         <v>303</v>
       </c>
-    </row>
-    <row r="3" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="13" t="s">
+      <c r="E5" s="13" t="s">
         <v>304</v>
       </c>
-      <c r="B3" s="13" t="s">
-        <v>21</v>
-      </c>
-      <c r="C3" s="13" t="s">
+    </row>
+    <row r="6" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="13" t="s">
         <v>305</v>
       </c>
-      <c r="D3" s="13" t="s">
+      <c r="B6" s="13" t="s">
+        <v>23</v>
+      </c>
+      <c r="C6" s="13" t="s">
         <v>306</v>
       </c>
-      <c r="E3" s="13" t="s">
+      <c r="D6" s="13" t="s">
         <v>307</v>
       </c>
-    </row>
-    <row r="4" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="13" t="s">
+      <c r="E6" s="13" t="s">
         <v>308</v>
       </c>
-      <c r="B4" s="13" t="s">
-        <v>23</v>
-      </c>
-      <c r="C4" s="13" t="s">
+    </row>
+    <row r="7" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="13" t="s">
         <v>309</v>
       </c>
-      <c r="D4" s="13" t="s">
+      <c r="B7" s="13" t="s">
+        <v>26</v>
+      </c>
+      <c r="C7" s="13" t="s">
         <v>310</v>
       </c>
-      <c r="E4" s="13" t="s">
+      <c r="D7" s="13" t="s">
         <v>311</v>
       </c>
-    </row>
-    <row r="5" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="13" t="s">
+      <c r="E7" s="13" t="s">
         <v>312</v>
       </c>
-      <c r="B5" s="13" t="s">
-        <v>26</v>
-      </c>
-      <c r="C5" s="13" t="s">
+    </row>
+    <row r="8" customFormat="false" ht="68.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="13" t="s">
         <v>313</v>
-      </c>
-      <c r="D5" s="13" t="s">
-        <v>314</v>
-      </c>
-      <c r="E5" s="13" t="s">
-        <v>315</v>
-      </c>
-    </row>
-    <row r="6" customFormat="false" ht="68.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="13" t="s">
-        <v>316</v>
-      </c>
-      <c r="B6" s="13" t="s">
-        <v>15</v>
-      </c>
-      <c r="C6" s="13" t="s">
-        <v>317</v>
-      </c>
-      <c r="D6" s="13" t="s">
-        <v>318</v>
-      </c>
-      <c r="E6" s="13" t="s">
-        <v>319</v>
-      </c>
-    </row>
-    <row r="7" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="13" t="s">
-        <v>320</v>
-      </c>
-      <c r="B7" s="13" t="s">
-        <v>15</v>
-      </c>
-      <c r="C7" s="13" t="s">
-        <v>321</v>
-      </c>
-      <c r="D7" s="13" t="s">
-        <v>322</v>
-      </c>
-      <c r="E7" s="13" t="s">
-        <v>323</v>
-      </c>
-    </row>
-    <row r="8" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="13" t="s">
-        <v>324</v>
       </c>
       <c r="B8" s="13" t="s">
         <v>15</v>
       </c>
       <c r="C8" s="13" t="s">
-        <v>325</v>
+        <v>314</v>
       </c>
       <c r="D8" s="13" t="s">
-        <v>326</v>
+        <v>315</v>
       </c>
       <c r="E8" s="13" t="s">
-        <v>327</v>
-      </c>
-    </row>
-    <row r="9" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>316</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="13" t="s">
-        <v>328</v>
+        <v>317</v>
       </c>
       <c r="B9" s="13" t="s">
-        <v>28</v>
+        <v>15</v>
       </c>
       <c r="C9" s="13" t="s">
-        <v>329</v>
+        <v>318</v>
       </c>
       <c r="D9" s="13" t="s">
-        <v>330</v>
+        <v>319</v>
       </c>
       <c r="E9" s="13" t="s">
-        <v>331</v>
-      </c>
-    </row>
-    <row r="10" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>320</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="13" t="s">
-        <v>332</v>
+        <v>321</v>
       </c>
       <c r="B10" s="13" t="s">
-        <v>28</v>
+        <v>15</v>
       </c>
       <c r="C10" s="13" t="s">
-        <v>333</v>
+        <v>322</v>
       </c>
       <c r="D10" s="13" t="s">
-        <v>334</v>
+        <v>323</v>
       </c>
       <c r="E10" s="13" t="s">
-        <v>335</v>
+        <v>324</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="13" t="s">
-        <v>336</v>
+        <v>325</v>
       </c>
       <c r="B11" s="13" t="s">
         <v>28</v>
       </c>
       <c r="C11" s="13" t="s">
-        <v>337</v>
+        <v>326</v>
       </c>
       <c r="D11" s="13" t="s">
-        <v>338</v>
+        <v>327</v>
       </c>
       <c r="E11" s="13" t="s">
-        <v>339</v>
-      </c>
-    </row>
-    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>328</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="13" t="s">
-        <v>340</v>
+        <v>329</v>
       </c>
       <c r="B12" s="13" t="s">
         <v>28</v>
       </c>
       <c r="C12" s="13" t="s">
+        <v>330</v>
+      </c>
+      <c r="D12" s="13" t="s">
+        <v>331</v>
+      </c>
+      <c r="E12" s="13" t="s">
+        <v>332</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="13" t="s">
+        <v>333</v>
+      </c>
+      <c r="B13" s="13" t="s">
+        <v>28</v>
+      </c>
+      <c r="C13" s="13" t="s">
+        <v>334</v>
+      </c>
+      <c r="D13" s="13" t="s">
+        <v>335</v>
+      </c>
+      <c r="E13" s="13" t="s">
+        <v>336</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A14" s="13" t="s">
+        <v>337</v>
+      </c>
+      <c r="B14" s="13" t="s">
+        <v>28</v>
+      </c>
+      <c r="C14" s="13" t="s">
+        <v>338</v>
+      </c>
+      <c r="D14" s="13" t="s">
+        <v>339</v>
+      </c>
+      <c r="E14" s="13" t="s">
+        <v>340</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A15" s="13" t="s">
         <v>341</v>
-      </c>
-      <c r="D12" s="13" t="s">
-        <v>342</v>
-      </c>
-      <c r="E12" s="13" t="s">
-        <v>343</v>
-      </c>
-    </row>
-    <row r="13" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="13" t="s">
-        <v>344</v>
-      </c>
-      <c r="B13" s="13" t="s">
-        <v>31</v>
-      </c>
-      <c r="C13" s="13" t="s">
-        <v>345</v>
-      </c>
-      <c r="D13" s="13" t="s">
-        <v>346</v>
-      </c>
-      <c r="E13" s="13" t="s">
-        <v>347</v>
-      </c>
-    </row>
-    <row r="14" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="13" t="s">
-        <v>348</v>
-      </c>
-      <c r="B14" s="13" t="s">
-        <v>31</v>
-      </c>
-      <c r="C14" s="13" t="s">
-        <v>349</v>
-      </c>
-      <c r="D14" s="13" t="s">
-        <v>350</v>
-      </c>
-      <c r="E14" s="13" t="s">
-        <v>351</v>
-      </c>
-    </row>
-    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="13" t="s">
-        <v>352</v>
       </c>
       <c r="B15" s="13" t="s">
         <v>31</v>
       </c>
       <c r="C15" s="13" t="s">
-        <v>353</v>
+        <v>342</v>
       </c>
       <c r="D15" s="13" t="s">
-        <v>354</v>
+        <v>343</v>
       </c>
       <c r="E15" s="13" t="s">
-        <v>355</v>
+        <v>344</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="13" t="s">
-        <v>356</v>
+        <v>345</v>
       </c>
       <c r="B16" s="13" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="C16" s="13" t="s">
-        <v>357</v>
+        <v>346</v>
       </c>
       <c r="D16" s="13" t="s">
-        <v>358</v>
+        <v>347</v>
       </c>
       <c r="E16" s="13" t="s">
-        <v>359</v>
-      </c>
-    </row>
-    <row r="17" customFormat="false" ht="68.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>348</v>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="13" t="s">
-        <v>360</v>
+        <v>349</v>
       </c>
       <c r="B17" s="13" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="C17" s="13" t="s">
-        <v>361</v>
+        <v>350</v>
       </c>
       <c r="D17" s="13" t="s">
-        <v>362</v>
+        <v>351</v>
       </c>
       <c r="E17" s="13" t="s">
-        <v>363</v>
-      </c>
-    </row>
-    <row r="18" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>352</v>
+      </c>
+    </row>
+    <row r="18" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="13" t="s">
-        <v>364</v>
+        <v>353</v>
       </c>
       <c r="B18" s="13" t="s">
         <v>32</v>
       </c>
       <c r="C18" s="13" t="s">
-        <v>365</v>
+        <v>354</v>
       </c>
       <c r="D18" s="13" t="s">
-        <v>366</v>
+        <v>355</v>
       </c>
       <c r="E18" s="13" t="s">
-        <v>367</v>
-      </c>
-    </row>
-    <row r="19" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>356</v>
+      </c>
+    </row>
+    <row r="19" customFormat="false" ht="68.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="13" t="s">
-        <v>368</v>
+        <v>357</v>
       </c>
       <c r="B19" s="13" t="s">
         <v>32</v>
       </c>
       <c r="C19" s="13" t="s">
-        <v>369</v>
+        <v>358</v>
       </c>
       <c r="D19" s="13" t="s">
-        <v>370</v>
+        <v>359</v>
       </c>
       <c r="E19" s="13" t="s">
-        <v>371</v>
-      </c>
-    </row>
-    <row r="20" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>360</v>
+      </c>
+    </row>
+    <row r="20" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="13" t="s">
-        <v>372</v>
+        <v>361</v>
       </c>
       <c r="B20" s="13" t="s">
         <v>32</v>
       </c>
       <c r="C20" s="13" t="s">
-        <v>373</v>
+        <v>362</v>
       </c>
       <c r="D20" s="13" t="s">
-        <v>374</v>
+        <v>363</v>
       </c>
       <c r="E20" s="13" t="s">
-        <v>375</v>
+        <v>364</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="13" t="s">
+        <v>365</v>
+      </c>
+      <c r="B21" s="13" t="s">
+        <v>32</v>
+      </c>
+      <c r="C21" s="13" t="s">
+        <v>366</v>
+      </c>
+      <c r="D21" s="13" t="s">
+        <v>367</v>
+      </c>
+      <c r="E21" s="13" t="s">
+        <v>368</v>
+      </c>
+    </row>
+    <row r="22" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A22" s="13" t="s">
+        <v>369</v>
+      </c>
+      <c r="B22" s="13" t="s">
+        <v>32</v>
+      </c>
+      <c r="C22" s="13" t="s">
+        <v>370</v>
+      </c>
+      <c r="D22" s="13" t="s">
+        <v>371</v>
+      </c>
+      <c r="E22" s="13" t="s">
+        <v>372</v>
+      </c>
+    </row>
+    <row r="23" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A23" s="13" t="s">
+        <v>373</v>
+      </c>
+      <c r="B23" s="13" t="s">
+        <v>374</v>
+      </c>
+      <c r="C23" s="13" t="s">
+        <v>375</v>
+      </c>
+      <c r="D23" s="13" t="s">
         <v>376</v>
       </c>
-      <c r="B21" s="13" t="s">
+      <c r="E23" s="13" t="s">
         <v>377</v>
       </c>
-      <c r="C21" s="13" t="s">
+    </row>
+    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A24" s="13" t="s">
         <v>378</v>
       </c>
-      <c r="D21" s="13" t="s">
+      <c r="B24" s="13" t="s">
+        <v>374</v>
+      </c>
+      <c r="C24" s="13" t="s">
         <v>379</v>
       </c>
-      <c r="E21" s="13" t="s">
+      <c r="D24" s="13" t="s">
         <v>380</v>
       </c>
-    </row>
-    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="13" t="s">
+      <c r="E24" s="13" t="s">
         <v>381</v>
       </c>
-      <c r="B22" s="13" t="s">
-        <v>377</v>
-      </c>
-      <c r="C22" s="13" t="s">
-        <v>382</v>
-      </c>
-      <c r="D22" s="13" t="s">
-        <v>383</v>
-      </c>
-      <c r="E22" s="13" t="s">
-        <v>384</v>
-      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:E22"/>
+  <autoFilter ref="A1:E24"/>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>

</xml_diff>

<commit_message>
Gap register Rev 4: correct licensing flag with verified GCCH SKU facts
Removes the incorrect verification question on the 55-seat tier: M365
Business Premium IS offered in GCC High (announced Nov 3; SKU stem
matches the quote), and the combined Defender + Purview Suite GCCH
add-on carries Entra ID P2, Defender for Endpoint P2, Defender for
Office 365 P2, and E5 Purview incl. Endpoint DLP - verified against
public documentation. Entra P2 now confirmed for all 150 users, so
G-06 drops to Medium with only third-party seats and overlap budget
remaining; Endpoint DLP licensing clause cleared from G-58. Still 41
open (26 High / 15 Medium) / 23 resolved.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01D9SFx2c7BjowTfENYrpiQo
</commit_message>
<xml_diff>
--- a/deliverables/WMP/WMP__Solution_Design_Gap_Register__20260824.xlsx
+++ b/deliverables/WMP/WMP__Solution_Design_Gap_Register__20260824.xlsx
@@ -31,7 +31,7 @@
     <t xml:space="preserve">WMP Solution Design — Inputs &amp; Decisions Gap Register</t>
   </si>
   <si>
-    <t xml:space="preserve">Rev 3 — updated 8/24/2026: join model, shop-floor MFA, and the licensing plan incorporated. Open questions only; resolved decisions on the 'Resolved Decisions' sheet.</t>
+    <t xml:space="preserve">Rev 4 — updated 8/24/2026: licensing plan verified against public GCC High SKU documentation (Business Premium GCCH + Defender/Purview Suite confirmed). Open questions only; resolved decisions on the 'Resolved Decisions' sheet.</t>
   </si>
   <si>
     <t xml:space="preserve">Wisconsin Metal Parts — Microsoft GCC High Migration (CMMC 2.0 Level 2)  |  Prepared by Essendis</t>
@@ -270,8 +270,7 @@
     <t xml:space="preserve">Half the controls in this design are SKU-dependent (PIM, risk policies, Defender for Endpoint, Purview labelling/DLP, audit retention); costing and configuration both stall until the SKU is fixed.</t>
   </si>
   <si>
-    <t xml:space="preserve">Confirm with the AOS-G partner that the 55-seat tier is a GCC High offering: the quote line reads 'M365 Business Premium' with no GCCH marker, and Business Premium has no native GCC High variant — verify what the paired 'BP Defender Purview Suite GCCH' actually delivers, specifically Entra ID P2 and Endpoint DLP entitlements for those 55 users.
-Who buys AvePoint Fly, ForensIT, and CallTower seats — WMP directly or through Essendis?
+    <t xml:space="preserve">Who buys AvePoint Fly, ForensIT, and CallTower seats — WMP directly or through Essendis?
 How long do commercial-tenant licences overlap GCC High, and is the overlap budgeted?</t>
   </si>
   <si>
@@ -282,7 +281,8 @@
 Teams Phone Standard GCCH x55 (RFT-00001-COMM)
 M365 F3 GCCH x80 (AAA-99952-COMM)
 M365 F5 Security + Compliance GCCH Add-on x80 (91Q-00003-COMM)
-= 150 users: 15 G5 / 55 BP tier / 80 F3 + F5 S&amp;C.</t>
+= 150 users: 15 G5 / 55 BP tier / 80 F3 + F5 S&amp;C.
+VERIFIED (public sources, 8/24): M365 Business Premium is offered in GCC High (announced Nov 3, ~300-seat cap; Microsoft SKU AAU-59343 matches the quote's AAD-59343 line). The combined Defender + Purview Suite GCCH add-on (AAV-01856 line) adds Entra ID P2, Defender for Endpoint P2, Defender for Office 365 P2, Defender for Identity/Cloud Apps, E5 Information Protection (auto-labeling, unified DLP incl. Endpoint DLP), Insider Risk, eDiscovery Premium, extended audit. With G5 (15) and F5 Security+Compliance (80), Entra ID P2 covers all 150 users; risk-based CA policies 7-8 are licensed tenant-wide.</t>
   </si>
   <si>
     <t xml:space="preserve">New section: M365 Design &gt; Licensing</t>
@@ -986,7 +986,7 @@
   <si>
     <t xml:space="preserve">Does the CUI label apply encryption and/or visual marking, or is it classification-only?
 Does DLP block on the CUI label alone (labeling is manual) or also on content detection? If content detection: provide WMP's CUI identifiers (part/contract/drawing numbers).
-Endpoint DLP (confirmed in scope): which restrictions — USB, print, clipboard — and is its licensing confirmed (ties to G-06)?</t>
+Endpoint DLP (in scope; licensing confirmed via the BP Defender/Purview suite and G5): which restrictions — USB, print, clipboard?</t>
   </si>
   <si>
     <t xml:space="preserve">WMP (8/24): CUI label is the only part of taxonomy in scope. Manual labeling. DLP should block. Endpoint DLP in scope. Communication compliance out of scope.</t>
@@ -1050,7 +1050,7 @@
     <t xml:space="preserve">Settled by the licensing plan: P2 arrives via M365 G5 (15 users) and the F5 Security + Compliance add-on (80 users); the 55-seat BP + Defender/Purview Suite tier's P2 entitlement is verified under G-06.</t>
   </si>
   <si>
-    <t xml:space="preserve">No separate purchase decision remains. Entra P2 coverage verification for the 55-seat tier is tracked in G-06.</t>
+    <t xml:space="preserve">No purchase decision remains: Entra ID P2 is confirmed licensed for all 150 users — G5 (15), BP + Defender/Purview Suite GCCH (55), F5 Security + Compliance add-on (80). Verified against public SKU documentation 8/24.</t>
   </si>
   <si>
     <t xml:space="preserve">G-09</t>
@@ -1502,24 +1502,28 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="17">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1527,7 +1531,7 @@
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1535,19 +1539,19 @@
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="165" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="165" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1871,251 +1875,251 @@
   <dimension ref="B2:F33"/>
   <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="2"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="40"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="14"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="4"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="26"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="2"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="40"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="4"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="26"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="14"/>
   </cols>
   <sheetData>
-    <row r="2" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B2" s="1" t="s">
+    <row r="2" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B2" s="2" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B3" s="2" t="s">
+    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B3" s="3" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B4" s="3" t="s">
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B4" s="4" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B6" s="4" t="s">
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B6" s="5" t="s">
         <v>3</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="57.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B7" s="5" t="s">
+      <c r="B7" s="6" t="s">
         <v>4</v>
       </c>
-      <c r="C7" s="5"/>
-      <c r="D7" s="5"/>
-      <c r="E7" s="5"/>
-      <c r="F7" s="5"/>
-    </row>
-    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B9" s="4" t="s">
+      <c r="C7" s="6"/>
+      <c r="D7" s="6"/>
+      <c r="E7" s="6"/>
+      <c r="F7" s="6"/>
+    </row>
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B9" s="5" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B10" s="6" t="s">
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B10" s="7" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B11" s="7" t="s">
+      <c r="B11" s="8" t="s">
         <v>7</v>
       </c>
-      <c r="C11" s="7"/>
-      <c r="D11" s="7"/>
-      <c r="E11" s="7"/>
-      <c r="F11" s="7"/>
-    </row>
-    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B13" s="6" t="s">
+      <c r="C11" s="8"/>
+      <c r="D11" s="8"/>
+      <c r="E11" s="8"/>
+      <c r="F11" s="8"/>
+    </row>
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B13" s="7" t="s">
         <v>8</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B14" s="7" t="s">
+      <c r="B14" s="8" t="s">
         <v>9</v>
       </c>
-      <c r="C14" s="7"/>
-      <c r="D14" s="7"/>
-      <c r="E14" s="7"/>
-      <c r="F14" s="7"/>
-    </row>
-    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B16" s="6" t="s">
+      <c r="C14" s="8"/>
+      <c r="D14" s="8"/>
+      <c r="E14" s="8"/>
+      <c r="F14" s="8"/>
+    </row>
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B16" s="7" t="s">
         <v>10</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B17" s="7" t="s">
+      <c r="B17" s="8" t="s">
         <v>11</v>
       </c>
-      <c r="C17" s="7"/>
-      <c r="D17" s="7"/>
-      <c r="E17" s="7"/>
-      <c r="F17" s="7"/>
-    </row>
-    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B19" s="4" t="s">
+      <c r="C17" s="8"/>
+      <c r="D17" s="8"/>
+      <c r="E17" s="8"/>
+      <c r="F17" s="8"/>
+    </row>
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B19" s="5" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B20" s="6" t="s">
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B20" s="7" t="s">
         <v>13</v>
       </c>
-      <c r="E20" s="6" t="s">
+      <c r="E20" s="7" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B21" s="8" t="s">
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B21" s="9" t="s">
         <v>15</v>
       </c>
-      <c r="C21" s="9" t="n">
+      <c r="C21" s="10" t="n">
         <f aca="false">COUNTIF('Gap Register'!B:B,B21)</f>
         <v>8</v>
       </c>
-      <c r="E21" s="8" t="s">
+      <c r="E21" s="9" t="s">
         <v>16</v>
       </c>
-      <c r="F21" s="9" t="n">
+      <c r="F21" s="10" t="n">
         <f aca="false">COUNTIF('Gap Register'!J:J,"High")</f>
-        <v>27</v>
-      </c>
-    </row>
-    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B22" s="8" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B22" s="9" t="s">
         <v>17</v>
       </c>
-      <c r="C22" s="9" t="n">
+      <c r="C22" s="10" t="n">
         <f aca="false">COUNTIF('Gap Register'!B:B,B22)</f>
         <v>3</v>
       </c>
-      <c r="E22" s="8" t="s">
+      <c r="E22" s="9" t="s">
         <v>18</v>
       </c>
-      <c r="F22" s="9" t="n">
+      <c r="F22" s="10" t="n">
         <f aca="false">COUNTIF('Gap Register'!J:J,"Medium")</f>
-        <v>14</v>
-      </c>
-    </row>
-    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B23" s="8" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B23" s="9" t="s">
         <v>19</v>
       </c>
-      <c r="C23" s="9" t="n">
+      <c r="C23" s="10" t="n">
         <f aca="false">COUNTIF('Gap Register'!B:B,B23)</f>
         <v>1</v>
       </c>
-      <c r="E23" s="8" t="s">
+      <c r="E23" s="9" t="s">
         <v>20</v>
       </c>
-      <c r="F23" s="9" t="n">
+      <c r="F23" s="10" t="n">
         <f aca="false">COUNTIF('Gap Register'!J:J,"Low")</f>
         <v>0</v>
       </c>
     </row>
-    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B24" s="8" t="s">
+    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B24" s="9" t="s">
         <v>21</v>
       </c>
-      <c r="C24" s="9" t="n">
+      <c r="C24" s="10" t="n">
         <f aca="false">COUNTIF('Gap Register'!B:B,B24)</f>
         <v>4</v>
       </c>
-      <c r="E24" s="10" t="s">
+      <c r="E24" s="11" t="s">
         <v>22</v>
       </c>
-      <c r="F24" s="11" t="n">
+      <c r="F24" s="12" t="n">
         <f aca="false">COUNTA('Gap Register'!A:A)-1</f>
         <v>41</v>
       </c>
     </row>
-    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B25" s="8" t="s">
+    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B25" s="9" t="s">
         <v>23</v>
       </c>
-      <c r="C25" s="9" t="n">
+      <c r="C25" s="10" t="n">
         <f aca="false">COUNTIF('Gap Register'!B:B,B25)</f>
         <v>3</v>
       </c>
-      <c r="E25" s="10" t="s">
+      <c r="E25" s="11" t="s">
         <v>24</v>
       </c>
-      <c r="F25" s="11" t="n">
+      <c r="F25" s="12" t="n">
         <f aca="false">COUNTA('Resolved Decisions'!A:A)-1</f>
         <v>23</v>
       </c>
     </row>
-    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B26" s="8" t="s">
+    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B26" s="9" t="s">
         <v>25</v>
       </c>
-      <c r="C26" s="9" t="n">
+      <c r="C26" s="10" t="n">
         <f aca="false">COUNTIF('Gap Register'!B:B,B26)</f>
         <v>3</v>
       </c>
     </row>
-    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B27" s="8" t="s">
+    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B27" s="9" t="s">
         <v>26</v>
       </c>
-      <c r="C27" s="9" t="n">
+      <c r="C27" s="10" t="n">
         <f aca="false">COUNTIF('Gap Register'!B:B,B27)</f>
         <v>2</v>
       </c>
     </row>
-    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B28" s="8" t="s">
+    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B28" s="9" t="s">
         <v>27</v>
       </c>
-      <c r="C28" s="9" t="n">
+      <c r="C28" s="10" t="n">
         <f aca="false">COUNTIF('Gap Register'!B:B,B28)</f>
         <v>4</v>
       </c>
     </row>
-    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B29" s="8" t="s">
+    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B29" s="9" t="s">
         <v>28</v>
       </c>
-      <c r="C29" s="9" t="n">
+      <c r="C29" s="10" t="n">
         <f aca="false">COUNTIF('Gap Register'!B:B,B29)</f>
         <v>4</v>
       </c>
     </row>
-    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B30" s="8" t="s">
+    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B30" s="9" t="s">
         <v>29</v>
       </c>
-      <c r="C30" s="9" t="n">
+      <c r="C30" s="10" t="n">
         <f aca="false">COUNTIF('Gap Register'!B:B,B30)</f>
         <v>3</v>
       </c>
     </row>
-    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B31" s="8" t="s">
+    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B31" s="9" t="s">
         <v>30</v>
       </c>
-      <c r="C31" s="9" t="n">
+      <c r="C31" s="10" t="n">
         <f aca="false">COUNTIF('Gap Register'!B:B,B31)</f>
         <v>2</v>
       </c>
     </row>
-    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B32" s="8" t="s">
+    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B32" s="9" t="s">
         <v>31</v>
       </c>
-      <c r="C32" s="9" t="n">
+      <c r="C32" s="10" t="n">
         <f aca="false">COUNTIF('Gap Register'!B:B,B32)</f>
         <v>2</v>
       </c>
     </row>
-    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B33" s="8" t="s">
+    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B33" s="9" t="s">
         <v>32</v>
       </c>
-      <c r="C33" s="9" t="n">
+      <c r="C33" s="10" t="n">
         <f aca="false">COUNTIF('Gap Register'!B:B,B33)</f>
         <v>2</v>
       </c>
@@ -2145,1460 +2149,1460 @@
   <dimension ref="A1:K42"/>
   <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="7"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="26"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="44"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="20"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="46"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="62"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="40"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="26"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="0" width="16"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="0" width="9"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="0" width="8"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="7"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="26"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="44"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="20"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="46"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="62"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="40"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="1" width="26"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="1" width="16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="1" width="9"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="1" width="8"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="12" t="s">
+    <row r="1" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A1" s="13" t="s">
         <v>33</v>
       </c>
-      <c r="B1" s="12" t="s">
+      <c r="B1" s="13" t="s">
         <v>34</v>
       </c>
-      <c r="C1" s="12" t="s">
+      <c r="C1" s="13" t="s">
         <v>35</v>
       </c>
-      <c r="D1" s="12" t="s">
+      <c r="D1" s="13" t="s">
         <v>6</v>
       </c>
-      <c r="E1" s="12" t="s">
+      <c r="E1" s="13" t="s">
         <v>36</v>
       </c>
-      <c r="F1" s="12" t="s">
+      <c r="F1" s="13" t="s">
         <v>37</v>
       </c>
-      <c r="G1" s="12" t="s">
+      <c r="G1" s="13" t="s">
         <v>38</v>
       </c>
-      <c r="H1" s="12" t="s">
+      <c r="H1" s="13" t="s">
         <v>39</v>
       </c>
-      <c r="I1" s="12" t="s">
+      <c r="I1" s="13" t="s">
         <v>10</v>
       </c>
-      <c r="J1" s="12" t="s">
+      <c r="J1" s="13" t="s">
         <v>8</v>
       </c>
-      <c r="K1" s="12" t="s">
+      <c r="K1" s="13" t="s">
         <v>40</v>
       </c>
     </row>
-    <row r="2" customFormat="false" ht="147" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="13" t="s">
+    <row r="2" customFormat="false" ht="147" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A2" s="14" t="s">
         <v>41</v>
       </c>
-      <c r="B2" s="13" t="s">
+      <c r="B2" s="14" t="s">
         <v>15</v>
       </c>
-      <c r="C2" s="13" t="s">
+      <c r="C2" s="14" t="s">
         <v>42</v>
       </c>
-      <c r="D2" s="13" t="s">
+      <c r="D2" s="14" t="s">
         <v>43</v>
       </c>
-      <c r="E2" s="13" t="s">
+      <c r="E2" s="14" t="s">
         <v>44</v>
       </c>
-      <c r="F2" s="13" t="s">
+      <c r="F2" s="14" t="s">
         <v>45</v>
       </c>
-      <c r="G2" s="13" t="s">
+      <c r="G2" s="14" t="s">
         <v>46</v>
       </c>
-      <c r="H2" s="13" t="s">
+      <c r="H2" s="14" t="s">
         <v>47</v>
       </c>
-      <c r="I2" s="13" t="s">
+      <c r="I2" s="14" t="s">
         <v>48</v>
       </c>
-      <c r="J2" s="14" t="s">
+      <c r="J2" s="15" t="s">
         <v>49</v>
       </c>
-      <c r="K2" s="13" t="s">
+      <c r="K2" s="14" t="s">
         <v>50</v>
       </c>
     </row>
-    <row r="3" customFormat="false" ht="79.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="13" t="s">
+    <row r="3" customFormat="false" ht="79.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A3" s="14" t="s">
         <v>51</v>
       </c>
-      <c r="B3" s="13" t="s">
+      <c r="B3" s="14" t="s">
         <v>17</v>
       </c>
-      <c r="C3" s="13" t="s">
+      <c r="C3" s="14" t="s">
         <v>52</v>
       </c>
-      <c r="D3" s="13" t="s">
+      <c r="D3" s="14" t="s">
         <v>53</v>
       </c>
-      <c r="E3" s="13" t="s">
+      <c r="E3" s="14" t="s">
         <v>54</v>
       </c>
-      <c r="F3" s="13" t="s">
+      <c r="F3" s="14" t="s">
         <v>55</v>
       </c>
-      <c r="G3" s="13"/>
-      <c r="H3" s="13" t="s">
+      <c r="G3" s="14"/>
+      <c r="H3" s="14" t="s">
         <v>56</v>
       </c>
-      <c r="I3" s="13" t="s">
+      <c r="I3" s="14" t="s">
         <v>57</v>
       </c>
-      <c r="J3" s="14" t="s">
+      <c r="J3" s="15" t="s">
         <v>49</v>
       </c>
-      <c r="K3" s="13" t="s">
+      <c r="K3" s="14" t="s">
         <v>50</v>
       </c>
     </row>
-    <row r="4" customFormat="false" ht="79.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="13" t="s">
+    <row r="4" customFormat="false" ht="79.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A4" s="14" t="s">
         <v>58</v>
       </c>
-      <c r="B4" s="13" t="s">
+      <c r="B4" s="14" t="s">
         <v>17</v>
       </c>
-      <c r="C4" s="13" t="s">
+      <c r="C4" s="14" t="s">
         <v>59</v>
       </c>
-      <c r="D4" s="13" t="s">
+      <c r="D4" s="14" t="s">
         <v>43</v>
       </c>
-      <c r="E4" s="13" t="s">
+      <c r="E4" s="14" t="s">
         <v>60</v>
       </c>
-      <c r="F4" s="13" t="s">
+      <c r="F4" s="14" t="s">
         <v>61</v>
       </c>
-      <c r="G4" s="13" t="s">
+      <c r="G4" s="14" t="s">
         <v>62</v>
       </c>
-      <c r="H4" s="13" t="s">
+      <c r="H4" s="14" t="s">
         <v>63</v>
       </c>
-      <c r="I4" s="13" t="s">
+      <c r="I4" s="14" t="s">
         <v>48</v>
       </c>
-      <c r="J4" s="15" t="s">
+      <c r="J4" s="16" t="s">
         <v>64</v>
       </c>
-      <c r="K4" s="13" t="s">
+      <c r="K4" s="14" t="s">
         <v>50</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="91" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="13" t="s">
+    <row r="5" customFormat="false" ht="90.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A5" s="14" t="s">
         <v>65</v>
       </c>
-      <c r="B5" s="13" t="s">
+      <c r="B5" s="14" t="s">
         <v>17</v>
       </c>
-      <c r="C5" s="13" t="s">
+      <c r="C5" s="14" t="s">
         <v>66</v>
       </c>
-      <c r="D5" s="13" t="s">
+      <c r="D5" s="14" t="s">
         <v>67</v>
       </c>
-      <c r="E5" s="13" t="s">
+      <c r="E5" s="14" t="s">
         <v>68</v>
       </c>
-      <c r="F5" s="13" t="s">
+      <c r="F5" s="14" t="s">
         <v>69</v>
       </c>
-      <c r="G5" s="13" t="s">
+      <c r="G5" s="14" t="s">
         <v>70</v>
       </c>
-      <c r="H5" s="13" t="s">
+      <c r="H5" s="14" t="s">
         <v>71</v>
       </c>
-      <c r="I5" s="13" t="s">
+      <c r="I5" s="14" t="s">
         <v>57</v>
       </c>
-      <c r="J5" s="14" t="s">
+      <c r="J5" s="15" t="s">
         <v>49</v>
       </c>
-      <c r="K5" s="13" t="s">
+      <c r="K5" s="14" t="s">
         <v>50</v>
       </c>
     </row>
-    <row r="6" customFormat="false" ht="113.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="13" t="s">
+    <row r="6" customFormat="false" ht="113.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A6" s="14" t="s">
         <v>72</v>
       </c>
-      <c r="B6" s="13" t="s">
+      <c r="B6" s="14" t="s">
         <v>19</v>
       </c>
-      <c r="C6" s="13" t="s">
+      <c r="C6" s="14" t="s">
         <v>73</v>
       </c>
-      <c r="D6" s="13" t="s">
+      <c r="D6" s="14" t="s">
         <v>74</v>
       </c>
-      <c r="E6" s="13" t="s">
+      <c r="E6" s="14" t="s">
         <v>75</v>
       </c>
-      <c r="F6" s="13" t="s">
+      <c r="F6" s="14" t="s">
         <v>76</v>
       </c>
-      <c r="G6" s="13" t="s">
+      <c r="G6" s="14" t="s">
         <v>77</v>
       </c>
-      <c r="H6" s="13" t="s">
+      <c r="H6" s="14" t="s">
         <v>78</v>
       </c>
-      <c r="I6" s="13" t="s">
+      <c r="I6" s="14" t="s">
         <v>57</v>
       </c>
-      <c r="J6" s="14" t="s">
+      <c r="J6" s="16" t="s">
+        <v>64</v>
+      </c>
+      <c r="K6" s="14" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="90.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A7" s="14" t="s">
+        <v>79</v>
+      </c>
+      <c r="B7" s="14" t="s">
+        <v>21</v>
+      </c>
+      <c r="C7" s="14" t="s">
+        <v>80</v>
+      </c>
+      <c r="D7" s="14" t="s">
+        <v>74</v>
+      </c>
+      <c r="E7" s="14" t="s">
+        <v>81</v>
+      </c>
+      <c r="F7" s="14" t="s">
+        <v>82</v>
+      </c>
+      <c r="G7" s="14" t="s">
+        <v>83</v>
+      </c>
+      <c r="H7" s="14" t="s">
+        <v>84</v>
+      </c>
+      <c r="I7" s="14" t="s">
+        <v>48</v>
+      </c>
+      <c r="J7" s="15" t="s">
         <v>49</v>
       </c>
-      <c r="K6" s="13" t="s">
+      <c r="K7" s="14" t="s">
         <v>50</v>
       </c>
     </row>
-    <row r="7" customFormat="false" ht="91" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="13" t="s">
-        <v>79</v>
-      </c>
-      <c r="B7" s="13" t="s">
+    <row r="8" customFormat="false" ht="68.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A8" s="14" t="s">
+        <v>85</v>
+      </c>
+      <c r="B8" s="14" t="s">
         <v>21</v>
       </c>
-      <c r="C7" s="13" t="s">
-        <v>80</v>
-      </c>
-      <c r="D7" s="13" t="s">
+      <c r="C8" s="14" t="s">
+        <v>86</v>
+      </c>
+      <c r="D8" s="14" t="s">
         <v>74</v>
       </c>
-      <c r="E7" s="13" t="s">
-        <v>81</v>
-      </c>
-      <c r="F7" s="13" t="s">
-        <v>82</v>
-      </c>
-      <c r="G7" s="13" t="s">
-        <v>83</v>
-      </c>
-      <c r="H7" s="13" t="s">
-        <v>84</v>
-      </c>
-      <c r="I7" s="13" t="s">
+      <c r="E8" s="14" t="s">
+        <v>87</v>
+      </c>
+      <c r="F8" s="14" t="s">
+        <v>88</v>
+      </c>
+      <c r="G8" s="14" t="s">
+        <v>89</v>
+      </c>
+      <c r="H8" s="14" t="s">
+        <v>90</v>
+      </c>
+      <c r="I8" s="14" t="s">
+        <v>57</v>
+      </c>
+      <c r="J8" s="16" t="s">
+        <v>64</v>
+      </c>
+      <c r="K8" s="14" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="57" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A9" s="14" t="s">
+        <v>91</v>
+      </c>
+      <c r="B9" s="14" t="s">
+        <v>21</v>
+      </c>
+      <c r="C9" s="14" t="s">
+        <v>92</v>
+      </c>
+      <c r="D9" s="14" t="s">
+        <v>74</v>
+      </c>
+      <c r="E9" s="14" t="s">
+        <v>93</v>
+      </c>
+      <c r="F9" s="14" t="s">
+        <v>94</v>
+      </c>
+      <c r="G9" s="14" t="s">
+        <v>95</v>
+      </c>
+      <c r="H9" s="14" t="s">
+        <v>96</v>
+      </c>
+      <c r="I9" s="14" t="s">
+        <v>57</v>
+      </c>
+      <c r="J9" s="16" t="s">
+        <v>64</v>
+      </c>
+      <c r="K9" s="14" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A10" s="14" t="s">
+        <v>97</v>
+      </c>
+      <c r="B10" s="14" t="s">
+        <v>21</v>
+      </c>
+      <c r="C10" s="14" t="s">
+        <v>98</v>
+      </c>
+      <c r="D10" s="14" t="s">
+        <v>53</v>
+      </c>
+      <c r="E10" s="14" t="s">
+        <v>99</v>
+      </c>
+      <c r="F10" s="14" t="s">
+        <v>100</v>
+      </c>
+      <c r="G10" s="14" t="s">
+        <v>101</v>
+      </c>
+      <c r="H10" s="14" t="s">
+        <v>102</v>
+      </c>
+      <c r="I10" s="14" t="s">
+        <v>57</v>
+      </c>
+      <c r="J10" s="16" t="s">
+        <v>64</v>
+      </c>
+      <c r="K10" s="14" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="57" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A11" s="14" t="s">
+        <v>103</v>
+      </c>
+      <c r="B11" s="14" t="s">
+        <v>23</v>
+      </c>
+      <c r="C11" s="14" t="s">
+        <v>104</v>
+      </c>
+      <c r="D11" s="14" t="s">
+        <v>74</v>
+      </c>
+      <c r="E11" s="14" t="s">
+        <v>105</v>
+      </c>
+      <c r="F11" s="14" t="s">
+        <v>106</v>
+      </c>
+      <c r="G11" s="14" t="s">
+        <v>107</v>
+      </c>
+      <c r="H11" s="14" t="s">
+        <v>108</v>
+      </c>
+      <c r="I11" s="14" t="s">
         <v>48</v>
       </c>
-      <c r="J7" s="14" t="s">
+      <c r="J11" s="16" t="s">
+        <v>64</v>
+      </c>
+      <c r="K11" s="14" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A12" s="14" t="s">
+        <v>109</v>
+      </c>
+      <c r="B12" s="14" t="s">
+        <v>23</v>
+      </c>
+      <c r="C12" s="14" t="s">
+        <v>110</v>
+      </c>
+      <c r="D12" s="14" t="s">
+        <v>53</v>
+      </c>
+      <c r="E12" s="14" t="s">
+        <v>111</v>
+      </c>
+      <c r="F12" s="14" t="s">
+        <v>112</v>
+      </c>
+      <c r="G12" s="14" t="s">
+        <v>113</v>
+      </c>
+      <c r="H12" s="14" t="s">
+        <v>114</v>
+      </c>
+      <c r="I12" s="14" t="s">
+        <v>115</v>
+      </c>
+      <c r="J12" s="15" t="s">
         <v>49</v>
       </c>
-      <c r="K7" s="13" t="s">
+      <c r="K12" s="14" t="s">
         <v>50</v>
       </c>
     </row>
-    <row r="8" customFormat="false" ht="68.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="13" t="s">
-        <v>85</v>
-      </c>
-      <c r="B8" s="13" t="s">
-        <v>21</v>
-      </c>
-      <c r="C8" s="13" t="s">
-        <v>86</v>
-      </c>
-      <c r="D8" s="13" t="s">
+    <row r="13" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A13" s="14" t="s">
+        <v>116</v>
+      </c>
+      <c r="B13" s="14" t="s">
+        <v>23</v>
+      </c>
+      <c r="C13" s="14" t="s">
+        <v>117</v>
+      </c>
+      <c r="D13" s="14" t="s">
         <v>74</v>
       </c>
-      <c r="E8" s="13" t="s">
-        <v>87</v>
-      </c>
-      <c r="F8" s="13" t="s">
-        <v>88</v>
-      </c>
-      <c r="G8" s="13" t="s">
-        <v>89</v>
-      </c>
-      <c r="H8" s="13" t="s">
-        <v>90</v>
-      </c>
-      <c r="I8" s="13" t="s">
+      <c r="E13" s="14" t="s">
+        <v>118</v>
+      </c>
+      <c r="F13" s="14" t="s">
+        <v>119</v>
+      </c>
+      <c r="G13" s="14" t="s">
+        <v>120</v>
+      </c>
+      <c r="H13" s="14" t="s">
+        <v>121</v>
+      </c>
+      <c r="I13" s="14" t="s">
         <v>57</v>
       </c>
-      <c r="J8" s="15" t="s">
+      <c r="J13" s="16" t="s">
         <v>64</v>
       </c>
-      <c r="K8" s="13" t="s">
+      <c r="K13" s="14" t="s">
         <v>50</v>
       </c>
     </row>
-    <row r="9" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="13" t="s">
-        <v>91</v>
-      </c>
-      <c r="B9" s="13" t="s">
-        <v>21</v>
-      </c>
-      <c r="C9" s="13" t="s">
-        <v>92</v>
-      </c>
-      <c r="D9" s="13" t="s">
+    <row r="14" customFormat="false" ht="124.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A14" s="14" t="s">
+        <v>122</v>
+      </c>
+      <c r="B14" s="14" t="s">
+        <v>25</v>
+      </c>
+      <c r="C14" s="14" t="s">
+        <v>123</v>
+      </c>
+      <c r="D14" s="14" t="s">
+        <v>67</v>
+      </c>
+      <c r="E14" s="14" t="s">
+        <v>124</v>
+      </c>
+      <c r="F14" s="14" t="s">
+        <v>125</v>
+      </c>
+      <c r="G14" s="14"/>
+      <c r="H14" s="14" t="s">
+        <v>126</v>
+      </c>
+      <c r="I14" s="14" t="s">
+        <v>57</v>
+      </c>
+      <c r="J14" s="15" t="s">
+        <v>49</v>
+      </c>
+      <c r="K14" s="14" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="68.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A15" s="14" t="s">
+        <v>127</v>
+      </c>
+      <c r="B15" s="14" t="s">
+        <v>25</v>
+      </c>
+      <c r="C15" s="14" t="s">
+        <v>128</v>
+      </c>
+      <c r="D15" s="14" t="s">
         <v>74</v>
       </c>
-      <c r="E9" s="13" t="s">
-        <v>93</v>
-      </c>
-      <c r="F9" s="13" t="s">
-        <v>94</v>
-      </c>
-      <c r="G9" s="13" t="s">
-        <v>95</v>
-      </c>
-      <c r="H9" s="13" t="s">
-        <v>96</v>
-      </c>
-      <c r="I9" s="13" t="s">
+      <c r="E15" s="14" t="s">
+        <v>129</v>
+      </c>
+      <c r="F15" s="14" t="s">
+        <v>130</v>
+      </c>
+      <c r="G15" s="14" t="s">
+        <v>131</v>
+      </c>
+      <c r="H15" s="14" t="s">
+        <v>132</v>
+      </c>
+      <c r="I15" s="14" t="s">
+        <v>48</v>
+      </c>
+      <c r="J15" s="16" t="s">
+        <v>64</v>
+      </c>
+      <c r="K15" s="14" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="90.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A16" s="14" t="s">
+        <v>133</v>
+      </c>
+      <c r="B16" s="14" t="s">
+        <v>25</v>
+      </c>
+      <c r="C16" s="14" t="s">
+        <v>134</v>
+      </c>
+      <c r="D16" s="14" t="s">
+        <v>53</v>
+      </c>
+      <c r="E16" s="14" t="s">
+        <v>135</v>
+      </c>
+      <c r="F16" s="14" t="s">
+        <v>136</v>
+      </c>
+      <c r="G16" s="14" t="s">
+        <v>137</v>
+      </c>
+      <c r="H16" s="14" t="s">
+        <v>138</v>
+      </c>
+      <c r="I16" s="14" t="s">
         <v>57</v>
       </c>
-      <c r="J9" s="15" t="s">
+      <c r="J16" s="16" t="s">
         <v>64</v>
       </c>
-      <c r="K9" s="13" t="s">
+      <c r="K16" s="14" t="s">
         <v>50</v>
       </c>
     </row>
-    <row r="10" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="13" t="s">
-        <v>97</v>
-      </c>
-      <c r="B10" s="13" t="s">
-        <v>21</v>
-      </c>
-      <c r="C10" s="13" t="s">
-        <v>98</v>
-      </c>
-      <c r="D10" s="13" t="s">
+    <row r="17" customFormat="false" ht="102" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A17" s="14" t="s">
+        <v>139</v>
+      </c>
+      <c r="B17" s="14" t="s">
+        <v>26</v>
+      </c>
+      <c r="C17" s="14" t="s">
+        <v>140</v>
+      </c>
+      <c r="D17" s="14" t="s">
+        <v>74</v>
+      </c>
+      <c r="E17" s="14" t="s">
+        <v>141</v>
+      </c>
+      <c r="F17" s="14" t="s">
+        <v>142</v>
+      </c>
+      <c r="G17" s="14"/>
+      <c r="H17" s="14" t="s">
+        <v>143</v>
+      </c>
+      <c r="I17" s="14" t="s">
+        <v>57</v>
+      </c>
+      <c r="J17" s="15" t="s">
+        <v>49</v>
+      </c>
+      <c r="K17" s="14" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="18" customFormat="false" ht="90.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A18" s="14" t="s">
+        <v>144</v>
+      </c>
+      <c r="B18" s="14" t="s">
+        <v>26</v>
+      </c>
+      <c r="C18" s="14" t="s">
+        <v>145</v>
+      </c>
+      <c r="D18" s="14" t="s">
         <v>53</v>
       </c>
-      <c r="E10" s="13" t="s">
-        <v>99</v>
-      </c>
-      <c r="F10" s="13" t="s">
-        <v>100</v>
-      </c>
-      <c r="G10" s="13" t="s">
-        <v>101</v>
-      </c>
-      <c r="H10" s="13" t="s">
-        <v>102</v>
-      </c>
-      <c r="I10" s="13" t="s">
+      <c r="E18" s="14" t="s">
+        <v>146</v>
+      </c>
+      <c r="F18" s="14" t="s">
+        <v>147</v>
+      </c>
+      <c r="G18" s="14" t="s">
+        <v>148</v>
+      </c>
+      <c r="H18" s="14" t="s">
+        <v>149</v>
+      </c>
+      <c r="I18" s="14" t="s">
         <v>57</v>
       </c>
-      <c r="J10" s="15" t="s">
+      <c r="J18" s="15" t="s">
+        <v>49</v>
+      </c>
+      <c r="K18" s="14" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="19" customFormat="false" ht="68.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A19" s="14" t="s">
+        <v>150</v>
+      </c>
+      <c r="B19" s="14" t="s">
+        <v>15</v>
+      </c>
+      <c r="C19" s="14" t="s">
+        <v>151</v>
+      </c>
+      <c r="D19" s="14" t="s">
+        <v>74</v>
+      </c>
+      <c r="E19" s="14" t="s">
+        <v>152</v>
+      </c>
+      <c r="F19" s="14" t="s">
+        <v>153</v>
+      </c>
+      <c r="G19" s="14" t="s">
+        <v>154</v>
+      </c>
+      <c r="H19" s="14" t="s">
+        <v>47</v>
+      </c>
+      <c r="I19" s="14" t="s">
+        <v>48</v>
+      </c>
+      <c r="J19" s="16" t="s">
         <v>64</v>
       </c>
-      <c r="K10" s="13" t="s">
+      <c r="K19" s="14" t="s">
         <v>50</v>
       </c>
     </row>
-    <row r="11" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="13" t="s">
-        <v>103</v>
-      </c>
-      <c r="B11" s="13" t="s">
-        <v>23</v>
-      </c>
-      <c r="C11" s="13" t="s">
-        <v>104</v>
-      </c>
-      <c r="D11" s="13" t="s">
+    <row r="20" customFormat="false" ht="90.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A20" s="14" t="s">
+        <v>155</v>
+      </c>
+      <c r="B20" s="14" t="s">
+        <v>15</v>
+      </c>
+      <c r="C20" s="14" t="s">
+        <v>156</v>
+      </c>
+      <c r="D20" s="14" t="s">
         <v>74</v>
       </c>
-      <c r="E11" s="13" t="s">
-        <v>105</v>
-      </c>
-      <c r="F11" s="13" t="s">
-        <v>106</v>
-      </c>
-      <c r="G11" s="13" t="s">
-        <v>107</v>
-      </c>
-      <c r="H11" s="13" t="s">
-        <v>108</v>
-      </c>
-      <c r="I11" s="13" t="s">
+      <c r="E20" s="14" t="s">
+        <v>157</v>
+      </c>
+      <c r="F20" s="14" t="s">
+        <v>158</v>
+      </c>
+      <c r="G20" s="14" t="s">
+        <v>159</v>
+      </c>
+      <c r="H20" s="14" t="s">
+        <v>160</v>
+      </c>
+      <c r="I20" s="14" t="s">
         <v>48</v>
       </c>
-      <c r="J11" s="15" t="s">
+      <c r="J20" s="15" t="s">
+        <v>49</v>
+      </c>
+      <c r="K20" s="14" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="21" customFormat="false" ht="102" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A21" s="14" t="s">
+        <v>161</v>
+      </c>
+      <c r="B21" s="14" t="s">
+        <v>15</v>
+      </c>
+      <c r="C21" s="14" t="s">
+        <v>162</v>
+      </c>
+      <c r="D21" s="14" t="s">
+        <v>53</v>
+      </c>
+      <c r="E21" s="14" t="s">
+        <v>163</v>
+      </c>
+      <c r="F21" s="14" t="s">
+        <v>164</v>
+      </c>
+      <c r="G21" s="14" t="s">
+        <v>165</v>
+      </c>
+      <c r="H21" s="14" t="s">
+        <v>166</v>
+      </c>
+      <c r="I21" s="14" t="s">
+        <v>57</v>
+      </c>
+      <c r="J21" s="15" t="s">
+        <v>49</v>
+      </c>
+      <c r="K21" s="14" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="22" customFormat="false" ht="102" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A22" s="14" t="s">
+        <v>167</v>
+      </c>
+      <c r="B22" s="14" t="s">
+        <v>15</v>
+      </c>
+      <c r="C22" s="14" t="s">
+        <v>168</v>
+      </c>
+      <c r="D22" s="14" t="s">
+        <v>74</v>
+      </c>
+      <c r="E22" s="14" t="s">
+        <v>169</v>
+      </c>
+      <c r="F22" s="14" t="s">
+        <v>170</v>
+      </c>
+      <c r="G22" s="14"/>
+      <c r="H22" s="14" t="s">
+        <v>171</v>
+      </c>
+      <c r="I22" s="14" t="s">
+        <v>57</v>
+      </c>
+      <c r="J22" s="15" t="s">
+        <v>49</v>
+      </c>
+      <c r="K22" s="14" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="23" customFormat="false" ht="90.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A23" s="14" t="s">
+        <v>172</v>
+      </c>
+      <c r="B23" s="14" t="s">
+        <v>15</v>
+      </c>
+      <c r="C23" s="14" t="s">
+        <v>173</v>
+      </c>
+      <c r="D23" s="14" t="s">
+        <v>53</v>
+      </c>
+      <c r="E23" s="14" t="s">
+        <v>174</v>
+      </c>
+      <c r="F23" s="14" t="s">
+        <v>175</v>
+      </c>
+      <c r="G23" s="14"/>
+      <c r="H23" s="14" t="s">
+        <v>176</v>
+      </c>
+      <c r="I23" s="14" t="s">
+        <v>57</v>
+      </c>
+      <c r="J23" s="15" t="s">
+        <v>49</v>
+      </c>
+      <c r="K23" s="14" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="24" customFormat="false" ht="68.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A24" s="14" t="s">
+        <v>177</v>
+      </c>
+      <c r="B24" s="14" t="s">
+        <v>15</v>
+      </c>
+      <c r="C24" s="14" t="s">
+        <v>178</v>
+      </c>
+      <c r="D24" s="14" t="s">
+        <v>53</v>
+      </c>
+      <c r="E24" s="14" t="s">
+        <v>179</v>
+      </c>
+      <c r="F24" s="14" t="s">
+        <v>180</v>
+      </c>
+      <c r="G24" s="14"/>
+      <c r="H24" s="14" t="s">
+        <v>181</v>
+      </c>
+      <c r="I24" s="14" t="s">
+        <v>115</v>
+      </c>
+      <c r="J24" s="16" t="s">
         <v>64</v>
       </c>
-      <c r="K11" s="13" t="s">
+      <c r="K24" s="14" t="s">
         <v>50</v>
       </c>
     </row>
-    <row r="12" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="13" t="s">
-        <v>109</v>
-      </c>
-      <c r="B12" s="13" t="s">
-        <v>23</v>
-      </c>
-      <c r="C12" s="13" t="s">
-        <v>110</v>
-      </c>
-      <c r="D12" s="13" t="s">
+    <row r="25" customFormat="false" ht="113.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A25" s="14" t="s">
+        <v>182</v>
+      </c>
+      <c r="B25" s="14" t="s">
+        <v>15</v>
+      </c>
+      <c r="C25" s="14" t="s">
+        <v>183</v>
+      </c>
+      <c r="D25" s="14" t="s">
+        <v>67</v>
+      </c>
+      <c r="E25" s="14" t="s">
+        <v>184</v>
+      </c>
+      <c r="F25" s="14" t="s">
+        <v>185</v>
+      </c>
+      <c r="G25" s="14"/>
+      <c r="H25" s="14" t="s">
+        <v>186</v>
+      </c>
+      <c r="I25" s="14" t="s">
+        <v>57</v>
+      </c>
+      <c r="J25" s="16" t="s">
+        <v>64</v>
+      </c>
+      <c r="K25" s="14" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="26" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A26" s="14" t="s">
+        <v>187</v>
+      </c>
+      <c r="B26" s="14" t="s">
+        <v>27</v>
+      </c>
+      <c r="C26" s="14" t="s">
+        <v>188</v>
+      </c>
+      <c r="D26" s="14" t="s">
+        <v>67</v>
+      </c>
+      <c r="E26" s="14" t="s">
+        <v>189</v>
+      </c>
+      <c r="F26" s="14" t="s">
+        <v>190</v>
+      </c>
+      <c r="G26" s="14" t="s">
+        <v>191</v>
+      </c>
+      <c r="H26" s="14" t="s">
+        <v>192</v>
+      </c>
+      <c r="I26" s="14" t="s">
+        <v>193</v>
+      </c>
+      <c r="J26" s="16" t="s">
+        <v>64</v>
+      </c>
+      <c r="K26" s="14" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="27" customFormat="false" ht="124.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A27" s="14" t="s">
+        <v>194</v>
+      </c>
+      <c r="B27" s="14" t="s">
+        <v>27</v>
+      </c>
+      <c r="C27" s="14" t="s">
+        <v>195</v>
+      </c>
+      <c r="D27" s="14" t="s">
         <v>53</v>
       </c>
-      <c r="E12" s="13" t="s">
-        <v>111</v>
-      </c>
-      <c r="F12" s="13" t="s">
-        <v>112</v>
-      </c>
-      <c r="G12" s="13" t="s">
-        <v>113</v>
-      </c>
-      <c r="H12" s="13" t="s">
-        <v>114</v>
-      </c>
-      <c r="I12" s="13" t="s">
+      <c r="E27" s="14" t="s">
+        <v>196</v>
+      </c>
+      <c r="F27" s="14" t="s">
+        <v>197</v>
+      </c>
+      <c r="G27" s="14" t="s">
+        <v>198</v>
+      </c>
+      <c r="H27" s="14" t="s">
+        <v>199</v>
+      </c>
+      <c r="I27" s="14" t="s">
+        <v>200</v>
+      </c>
+      <c r="J27" s="15" t="s">
+        <v>49</v>
+      </c>
+      <c r="K27" s="14" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="28" customFormat="false" ht="102" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A28" s="14" t="s">
+        <v>201</v>
+      </c>
+      <c r="B28" s="14" t="s">
+        <v>27</v>
+      </c>
+      <c r="C28" s="14" t="s">
+        <v>202</v>
+      </c>
+      <c r="D28" s="14" t="s">
+        <v>53</v>
+      </c>
+      <c r="E28" s="14" t="s">
+        <v>203</v>
+      </c>
+      <c r="F28" s="14" t="s">
+        <v>204</v>
+      </c>
+      <c r="G28" s="14"/>
+      <c r="H28" s="14" t="s">
+        <v>205</v>
+      </c>
+      <c r="I28" s="14" t="s">
+        <v>200</v>
+      </c>
+      <c r="J28" s="15" t="s">
+        <v>49</v>
+      </c>
+      <c r="K28" s="14" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="29" customFormat="false" ht="102" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A29" s="14" t="s">
+        <v>206</v>
+      </c>
+      <c r="B29" s="14" t="s">
+        <v>27</v>
+      </c>
+      <c r="C29" s="14" t="s">
+        <v>207</v>
+      </c>
+      <c r="D29" s="14" t="s">
+        <v>53</v>
+      </c>
+      <c r="E29" s="14" t="s">
+        <v>208</v>
+      </c>
+      <c r="F29" s="14" t="s">
+        <v>209</v>
+      </c>
+      <c r="G29" s="14"/>
+      <c r="H29" s="14" t="s">
+        <v>210</v>
+      </c>
+      <c r="I29" s="14" t="s">
+        <v>200</v>
+      </c>
+      <c r="J29" s="15" t="s">
+        <v>49</v>
+      </c>
+      <c r="K29" s="14" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="30" customFormat="false" ht="113.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A30" s="14" t="s">
+        <v>211</v>
+      </c>
+      <c r="B30" s="14" t="s">
+        <v>28</v>
+      </c>
+      <c r="C30" s="14" t="s">
+        <v>212</v>
+      </c>
+      <c r="D30" s="14" t="s">
+        <v>53</v>
+      </c>
+      <c r="E30" s="14" t="s">
+        <v>213</v>
+      </c>
+      <c r="F30" s="14" t="s">
+        <v>214</v>
+      </c>
+      <c r="G30" s="14" t="s">
+        <v>215</v>
+      </c>
+      <c r="H30" s="14" t="s">
+        <v>216</v>
+      </c>
+      <c r="I30" s="14" t="s">
+        <v>57</v>
+      </c>
+      <c r="J30" s="15" t="s">
+        <v>49</v>
+      </c>
+      <c r="K30" s="14" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="31" customFormat="false" ht="79.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A31" s="14" t="s">
+        <v>217</v>
+      </c>
+      <c r="B31" s="14" t="s">
+        <v>28</v>
+      </c>
+      <c r="C31" s="14" t="s">
+        <v>218</v>
+      </c>
+      <c r="D31" s="14" t="s">
+        <v>74</v>
+      </c>
+      <c r="E31" s="14" t="s">
+        <v>219</v>
+      </c>
+      <c r="F31" s="14" t="s">
+        <v>220</v>
+      </c>
+      <c r="G31" s="14" t="s">
+        <v>221</v>
+      </c>
+      <c r="H31" s="14" t="s">
+        <v>222</v>
+      </c>
+      <c r="I31" s="14" t="s">
+        <v>57</v>
+      </c>
+      <c r="J31" s="15" t="s">
+        <v>49</v>
+      </c>
+      <c r="K31" s="14" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="32" customFormat="false" ht="79.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A32" s="14" t="s">
+        <v>223</v>
+      </c>
+      <c r="B32" s="14" t="s">
+        <v>28</v>
+      </c>
+      <c r="C32" s="14" t="s">
+        <v>224</v>
+      </c>
+      <c r="D32" s="14" t="s">
+        <v>53</v>
+      </c>
+      <c r="E32" s="14" t="s">
+        <v>225</v>
+      </c>
+      <c r="F32" s="14" t="s">
+        <v>226</v>
+      </c>
+      <c r="G32" s="14"/>
+      <c r="H32" s="14" t="s">
+        <v>227</v>
+      </c>
+      <c r="I32" s="14" t="s">
+        <v>57</v>
+      </c>
+      <c r="J32" s="15" t="s">
+        <v>49</v>
+      </c>
+      <c r="K32" s="14" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="33" customFormat="false" ht="57" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A33" s="14" t="s">
+        <v>228</v>
+      </c>
+      <c r="B33" s="14" t="s">
+        <v>28</v>
+      </c>
+      <c r="C33" s="14" t="s">
+        <v>229</v>
+      </c>
+      <c r="D33" s="14" t="s">
+        <v>74</v>
+      </c>
+      <c r="E33" s="14" t="s">
+        <v>230</v>
+      </c>
+      <c r="F33" s="14" t="s">
+        <v>231</v>
+      </c>
+      <c r="G33" s="14" t="s">
+        <v>232</v>
+      </c>
+      <c r="H33" s="14" t="s">
+        <v>233</v>
+      </c>
+      <c r="I33" s="14" t="s">
+        <v>57</v>
+      </c>
+      <c r="J33" s="16" t="s">
+        <v>64</v>
+      </c>
+      <c r="K33" s="14" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="34" customFormat="false" ht="79.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A34" s="14" t="s">
+        <v>234</v>
+      </c>
+      <c r="B34" s="14" t="s">
+        <v>29</v>
+      </c>
+      <c r="C34" s="14" t="s">
+        <v>235</v>
+      </c>
+      <c r="D34" s="14" t="s">
+        <v>53</v>
+      </c>
+      <c r="E34" s="14" t="s">
+        <v>236</v>
+      </c>
+      <c r="F34" s="14" t="s">
+        <v>237</v>
+      </c>
+      <c r="G34" s="14" t="s">
+        <v>238</v>
+      </c>
+      <c r="H34" s="14" t="s">
+        <v>239</v>
+      </c>
+      <c r="I34" s="14" t="s">
         <v>115</v>
       </c>
-      <c r="J12" s="14" t="s">
+      <c r="J34" s="15" t="s">
         <v>49</v>
       </c>
-      <c r="K12" s="13" t="s">
+      <c r="K34" s="14" t="s">
         <v>50</v>
       </c>
     </row>
-    <row r="13" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="13" t="s">
-        <v>116</v>
-      </c>
-      <c r="B13" s="13" t="s">
-        <v>23</v>
-      </c>
-      <c r="C13" s="13" t="s">
-        <v>117</v>
-      </c>
-      <c r="D13" s="13" t="s">
+    <row r="35" customFormat="false" ht="124.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A35" s="14" t="s">
+        <v>240</v>
+      </c>
+      <c r="B35" s="14" t="s">
+        <v>29</v>
+      </c>
+      <c r="C35" s="14" t="s">
+        <v>241</v>
+      </c>
+      <c r="D35" s="14" t="s">
         <v>74</v>
       </c>
-      <c r="E13" s="13" t="s">
-        <v>118</v>
-      </c>
-      <c r="F13" s="13" t="s">
-        <v>119</v>
-      </c>
-      <c r="G13" s="13" t="s">
-        <v>120</v>
-      </c>
-      <c r="H13" s="13" t="s">
-        <v>121</v>
-      </c>
-      <c r="I13" s="13" t="s">
+      <c r="E35" s="14" t="s">
+        <v>242</v>
+      </c>
+      <c r="F35" s="14" t="s">
+        <v>243</v>
+      </c>
+      <c r="G35" s="14"/>
+      <c r="H35" s="14" t="s">
+        <v>244</v>
+      </c>
+      <c r="I35" s="14" t="s">
+        <v>48</v>
+      </c>
+      <c r="J35" s="15" t="s">
+        <v>49</v>
+      </c>
+      <c r="K35" s="14" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="36" customFormat="false" ht="102" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A36" s="14" t="s">
+        <v>245</v>
+      </c>
+      <c r="B36" s="14" t="s">
+        <v>29</v>
+      </c>
+      <c r="C36" s="14" t="s">
+        <v>246</v>
+      </c>
+      <c r="D36" s="14" t="s">
+        <v>74</v>
+      </c>
+      <c r="E36" s="14" t="s">
+        <v>247</v>
+      </c>
+      <c r="F36" s="14" t="s">
+        <v>248</v>
+      </c>
+      <c r="G36" s="14" t="s">
+        <v>249</v>
+      </c>
+      <c r="H36" s="14" t="s">
+        <v>250</v>
+      </c>
+      <c r="I36" s="14" t="s">
         <v>57</v>
       </c>
-      <c r="J13" s="15" t="s">
+      <c r="J36" s="15" t="s">
+        <v>49</v>
+      </c>
+      <c r="K36" s="14" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="37" customFormat="false" ht="79.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A37" s="14" t="s">
+        <v>251</v>
+      </c>
+      <c r="B37" s="14" t="s">
+        <v>30</v>
+      </c>
+      <c r="C37" s="14" t="s">
+        <v>252</v>
+      </c>
+      <c r="D37" s="14" t="s">
+        <v>74</v>
+      </c>
+      <c r="E37" s="14" t="s">
+        <v>253</v>
+      </c>
+      <c r="F37" s="14" t="s">
+        <v>254</v>
+      </c>
+      <c r="G37" s="14"/>
+      <c r="H37" s="14" t="s">
+        <v>255</v>
+      </c>
+      <c r="I37" s="14" t="s">
+        <v>57</v>
+      </c>
+      <c r="J37" s="15" t="s">
+        <v>49</v>
+      </c>
+      <c r="K37" s="14" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="38" customFormat="false" ht="102" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A38" s="14" t="s">
+        <v>256</v>
+      </c>
+      <c r="B38" s="14" t="s">
+        <v>30</v>
+      </c>
+      <c r="C38" s="14" t="s">
+        <v>257</v>
+      </c>
+      <c r="D38" s="14" t="s">
+        <v>74</v>
+      </c>
+      <c r="E38" s="14" t="s">
+        <v>258</v>
+      </c>
+      <c r="F38" s="14" t="s">
+        <v>259</v>
+      </c>
+      <c r="G38" s="14"/>
+      <c r="H38" s="14" t="s">
+        <v>260</v>
+      </c>
+      <c r="I38" s="14" t="s">
+        <v>57</v>
+      </c>
+      <c r="J38" s="16" t="s">
         <v>64</v>
       </c>
-      <c r="K13" s="13" t="s">
+      <c r="K38" s="14" t="s">
         <v>50</v>
       </c>
     </row>
-    <row r="14" customFormat="false" ht="124.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="13" t="s">
-        <v>122</v>
-      </c>
-      <c r="B14" s="13" t="s">
-        <v>25</v>
-      </c>
-      <c r="C14" s="13" t="s">
-        <v>123</v>
-      </c>
-      <c r="D14" s="13" t="s">
+    <row r="39" customFormat="false" ht="90.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A39" s="14" t="s">
+        <v>261</v>
+      </c>
+      <c r="B39" s="14" t="s">
+        <v>31</v>
+      </c>
+      <c r="C39" s="14" t="s">
+        <v>262</v>
+      </c>
+      <c r="D39" s="14" t="s">
         <v>67</v>
       </c>
-      <c r="E14" s="13" t="s">
-        <v>124</v>
-      </c>
-      <c r="F14" s="13" t="s">
-        <v>125</v>
-      </c>
-      <c r="G14" s="13"/>
-      <c r="H14" s="13" t="s">
-        <v>126</v>
-      </c>
-      <c r="I14" s="13" t="s">
+      <c r="E39" s="14" t="s">
+        <v>263</v>
+      </c>
+      <c r="F39" s="14" t="s">
+        <v>264</v>
+      </c>
+      <c r="G39" s="14" t="s">
+        <v>265</v>
+      </c>
+      <c r="H39" s="14" t="s">
+        <v>266</v>
+      </c>
+      <c r="I39" s="14" t="s">
         <v>57</v>
       </c>
-      <c r="J14" s="14" t="s">
+      <c r="J39" s="15" t="s">
         <v>49</v>
       </c>
-      <c r="K14" s="13" t="s">
+      <c r="K39" s="14" t="s">
         <v>50</v>
       </c>
     </row>
-    <row r="15" customFormat="false" ht="68.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="13" t="s">
-        <v>127</v>
-      </c>
-      <c r="B15" s="13" t="s">
-        <v>25</v>
-      </c>
-      <c r="C15" s="13" t="s">
-        <v>128</v>
-      </c>
-      <c r="D15" s="13" t="s">
+    <row r="40" customFormat="false" ht="90.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A40" s="14" t="s">
+        <v>267</v>
+      </c>
+      <c r="B40" s="14" t="s">
+        <v>31</v>
+      </c>
+      <c r="C40" s="14" t="s">
+        <v>268</v>
+      </c>
+      <c r="D40" s="14" t="s">
         <v>74</v>
       </c>
-      <c r="E15" s="13" t="s">
-        <v>129</v>
-      </c>
-      <c r="F15" s="13" t="s">
-        <v>130</v>
-      </c>
-      <c r="G15" s="13" t="s">
-        <v>131</v>
-      </c>
-      <c r="H15" s="13" t="s">
-        <v>132</v>
-      </c>
-      <c r="I15" s="13" t="s">
-        <v>48</v>
-      </c>
-      <c r="J15" s="15" t="s">
-        <v>64</v>
-      </c>
-      <c r="K15" s="13" t="s">
+      <c r="E40" s="14" t="s">
+        <v>269</v>
+      </c>
+      <c r="F40" s="14" t="s">
+        <v>270</v>
+      </c>
+      <c r="G40" s="14" t="s">
+        <v>271</v>
+      </c>
+      <c r="H40" s="14" t="s">
+        <v>272</v>
+      </c>
+      <c r="I40" s="14" t="s">
+        <v>57</v>
+      </c>
+      <c r="J40" s="15" t="s">
+        <v>49</v>
+      </c>
+      <c r="K40" s="14" t="s">
         <v>50</v>
       </c>
     </row>
-    <row r="16" customFormat="false" ht="91" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="13" t="s">
-        <v>133</v>
-      </c>
-      <c r="B16" s="13" t="s">
-        <v>25</v>
-      </c>
-      <c r="C16" s="13" t="s">
-        <v>134</v>
-      </c>
-      <c r="D16" s="13" t="s">
-        <v>53</v>
-      </c>
-      <c r="E16" s="13" t="s">
-        <v>135</v>
-      </c>
-      <c r="F16" s="13" t="s">
-        <v>136</v>
-      </c>
-      <c r="G16" s="13" t="s">
-        <v>137</v>
-      </c>
-      <c r="H16" s="13" t="s">
-        <v>138</v>
-      </c>
-      <c r="I16" s="13" t="s">
+    <row r="41" customFormat="false" ht="57" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A41" s="14" t="s">
+        <v>273</v>
+      </c>
+      <c r="B41" s="14" t="s">
+        <v>32</v>
+      </c>
+      <c r="C41" s="14" t="s">
+        <v>274</v>
+      </c>
+      <c r="D41" s="14" t="s">
+        <v>74</v>
+      </c>
+      <c r="E41" s="14" t="s">
+        <v>275</v>
+      </c>
+      <c r="F41" s="14" t="s">
+        <v>276</v>
+      </c>
+      <c r="G41" s="14" t="s">
+        <v>277</v>
+      </c>
+      <c r="H41" s="14" t="s">
+        <v>278</v>
+      </c>
+      <c r="I41" s="14" t="s">
         <v>57</v>
       </c>
-      <c r="J16" s="15" t="s">
-        <v>64</v>
-      </c>
-      <c r="K16" s="13" t="s">
+      <c r="J41" s="15" t="s">
+        <v>49</v>
+      </c>
+      <c r="K41" s="14" t="s">
         <v>50</v>
       </c>
     </row>
-    <row r="17" customFormat="false" ht="102.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="13" t="s">
-        <v>139</v>
-      </c>
-      <c r="B17" s="13" t="s">
-        <v>26</v>
-      </c>
-      <c r="C17" s="13" t="s">
-        <v>140</v>
-      </c>
-      <c r="D17" s="13" t="s">
+    <row r="42" customFormat="false" ht="102" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A42" s="14" t="s">
+        <v>279</v>
+      </c>
+      <c r="B42" s="14" t="s">
+        <v>32</v>
+      </c>
+      <c r="C42" s="14" t="s">
+        <v>280</v>
+      </c>
+      <c r="D42" s="14" t="s">
         <v>74</v>
       </c>
-      <c r="E17" s="13" t="s">
-        <v>141</v>
-      </c>
-      <c r="F17" s="13" t="s">
-        <v>142</v>
-      </c>
-      <c r="G17" s="13"/>
-      <c r="H17" s="13" t="s">
-        <v>143</v>
-      </c>
-      <c r="I17" s="13" t="s">
-        <v>57</v>
-      </c>
-      <c r="J17" s="14" t="s">
+      <c r="E42" s="14" t="s">
+        <v>281</v>
+      </c>
+      <c r="F42" s="14" t="s">
+        <v>282</v>
+      </c>
+      <c r="G42" s="14" t="s">
+        <v>283</v>
+      </c>
+      <c r="H42" s="14" t="s">
+        <v>284</v>
+      </c>
+      <c r="I42" s="14" t="s">
+        <v>285</v>
+      </c>
+      <c r="J42" s="15" t="s">
         <v>49</v>
       </c>
-      <c r="K17" s="13" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="18" customFormat="false" ht="91" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="13" t="s">
-        <v>144</v>
-      </c>
-      <c r="B18" s="13" t="s">
-        <v>26</v>
-      </c>
-      <c r="C18" s="13" t="s">
-        <v>145</v>
-      </c>
-      <c r="D18" s="13" t="s">
-        <v>53</v>
-      </c>
-      <c r="E18" s="13" t="s">
-        <v>146</v>
-      </c>
-      <c r="F18" s="13" t="s">
-        <v>147</v>
-      </c>
-      <c r="G18" s="13" t="s">
-        <v>148</v>
-      </c>
-      <c r="H18" s="13" t="s">
-        <v>149</v>
-      </c>
-      <c r="I18" s="13" t="s">
-        <v>57</v>
-      </c>
-      <c r="J18" s="14" t="s">
-        <v>49</v>
-      </c>
-      <c r="K18" s="13" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="19" customFormat="false" ht="68.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="13" t="s">
-        <v>150</v>
-      </c>
-      <c r="B19" s="13" t="s">
-        <v>15</v>
-      </c>
-      <c r="C19" s="13" t="s">
-        <v>151</v>
-      </c>
-      <c r="D19" s="13" t="s">
-        <v>74</v>
-      </c>
-      <c r="E19" s="13" t="s">
-        <v>152</v>
-      </c>
-      <c r="F19" s="13" t="s">
-        <v>153</v>
-      </c>
-      <c r="G19" s="13" t="s">
-        <v>154</v>
-      </c>
-      <c r="H19" s="13" t="s">
-        <v>47</v>
-      </c>
-      <c r="I19" s="13" t="s">
-        <v>48</v>
-      </c>
-      <c r="J19" s="15" t="s">
-        <v>64</v>
-      </c>
-      <c r="K19" s="13" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="20" customFormat="false" ht="91" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="13" t="s">
-        <v>155</v>
-      </c>
-      <c r="B20" s="13" t="s">
-        <v>15</v>
-      </c>
-      <c r="C20" s="13" t="s">
-        <v>156</v>
-      </c>
-      <c r="D20" s="13" t="s">
-        <v>74</v>
-      </c>
-      <c r="E20" s="13" t="s">
-        <v>157</v>
-      </c>
-      <c r="F20" s="13" t="s">
-        <v>158</v>
-      </c>
-      <c r="G20" s="13" t="s">
-        <v>159</v>
-      </c>
-      <c r="H20" s="13" t="s">
-        <v>160</v>
-      </c>
-      <c r="I20" s="13" t="s">
-        <v>48</v>
-      </c>
-      <c r="J20" s="14" t="s">
-        <v>49</v>
-      </c>
-      <c r="K20" s="13" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="21" customFormat="false" ht="102.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="13" t="s">
-        <v>161</v>
-      </c>
-      <c r="B21" s="13" t="s">
-        <v>15</v>
-      </c>
-      <c r="C21" s="13" t="s">
-        <v>162</v>
-      </c>
-      <c r="D21" s="13" t="s">
-        <v>53</v>
-      </c>
-      <c r="E21" s="13" t="s">
-        <v>163</v>
-      </c>
-      <c r="F21" s="13" t="s">
-        <v>164</v>
-      </c>
-      <c r="G21" s="13" t="s">
-        <v>165</v>
-      </c>
-      <c r="H21" s="13" t="s">
-        <v>166</v>
-      </c>
-      <c r="I21" s="13" t="s">
-        <v>57</v>
-      </c>
-      <c r="J21" s="14" t="s">
-        <v>49</v>
-      </c>
-      <c r="K21" s="13" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="22" customFormat="false" ht="102.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="13" t="s">
-        <v>167</v>
-      </c>
-      <c r="B22" s="13" t="s">
-        <v>15</v>
-      </c>
-      <c r="C22" s="13" t="s">
-        <v>168</v>
-      </c>
-      <c r="D22" s="13" t="s">
-        <v>74</v>
-      </c>
-      <c r="E22" s="13" t="s">
-        <v>169</v>
-      </c>
-      <c r="F22" s="13" t="s">
-        <v>170</v>
-      </c>
-      <c r="G22" s="13"/>
-      <c r="H22" s="13" t="s">
-        <v>171</v>
-      </c>
-      <c r="I22" s="13" t="s">
-        <v>57</v>
-      </c>
-      <c r="J22" s="14" t="s">
-        <v>49</v>
-      </c>
-      <c r="K22" s="13" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="23" customFormat="false" ht="91" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="13" t="s">
-        <v>172</v>
-      </c>
-      <c r="B23" s="13" t="s">
-        <v>15</v>
-      </c>
-      <c r="C23" s="13" t="s">
-        <v>173</v>
-      </c>
-      <c r="D23" s="13" t="s">
-        <v>53</v>
-      </c>
-      <c r="E23" s="13" t="s">
-        <v>174</v>
-      </c>
-      <c r="F23" s="13" t="s">
-        <v>175</v>
-      </c>
-      <c r="G23" s="13"/>
-      <c r="H23" s="13" t="s">
-        <v>176</v>
-      </c>
-      <c r="I23" s="13" t="s">
-        <v>57</v>
-      </c>
-      <c r="J23" s="14" t="s">
-        <v>49</v>
-      </c>
-      <c r="K23" s="13" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="24" customFormat="false" ht="68.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="13" t="s">
-        <v>177</v>
-      </c>
-      <c r="B24" s="13" t="s">
-        <v>15</v>
-      </c>
-      <c r="C24" s="13" t="s">
-        <v>178</v>
-      </c>
-      <c r="D24" s="13" t="s">
-        <v>53</v>
-      </c>
-      <c r="E24" s="13" t="s">
-        <v>179</v>
-      </c>
-      <c r="F24" s="13" t="s">
-        <v>180</v>
-      </c>
-      <c r="G24" s="13"/>
-      <c r="H24" s="13" t="s">
-        <v>181</v>
-      </c>
-      <c r="I24" s="13" t="s">
-        <v>115</v>
-      </c>
-      <c r="J24" s="15" t="s">
-        <v>64</v>
-      </c>
-      <c r="K24" s="13" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="25" customFormat="false" ht="113.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A25" s="13" t="s">
-        <v>182</v>
-      </c>
-      <c r="B25" s="13" t="s">
-        <v>15</v>
-      </c>
-      <c r="C25" s="13" t="s">
-        <v>183</v>
-      </c>
-      <c r="D25" s="13" t="s">
-        <v>67</v>
-      </c>
-      <c r="E25" s="13" t="s">
-        <v>184</v>
-      </c>
-      <c r="F25" s="13" t="s">
-        <v>185</v>
-      </c>
-      <c r="G25" s="13"/>
-      <c r="H25" s="13" t="s">
-        <v>186</v>
-      </c>
-      <c r="I25" s="13" t="s">
-        <v>57</v>
-      </c>
-      <c r="J25" s="15" t="s">
-        <v>64</v>
-      </c>
-      <c r="K25" s="13" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="26" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A26" s="13" t="s">
-        <v>187</v>
-      </c>
-      <c r="B26" s="13" t="s">
-        <v>27</v>
-      </c>
-      <c r="C26" s="13" t="s">
-        <v>188</v>
-      </c>
-      <c r="D26" s="13" t="s">
-        <v>67</v>
-      </c>
-      <c r="E26" s="13" t="s">
-        <v>189</v>
-      </c>
-      <c r="F26" s="13" t="s">
-        <v>190</v>
-      </c>
-      <c r="G26" s="13" t="s">
-        <v>191</v>
-      </c>
-      <c r="H26" s="13" t="s">
-        <v>192</v>
-      </c>
-      <c r="I26" s="13" t="s">
-        <v>193</v>
-      </c>
-      <c r="J26" s="15" t="s">
-        <v>64</v>
-      </c>
-      <c r="K26" s="13" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="27" customFormat="false" ht="124.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A27" s="13" t="s">
-        <v>194</v>
-      </c>
-      <c r="B27" s="13" t="s">
-        <v>27</v>
-      </c>
-      <c r="C27" s="13" t="s">
-        <v>195</v>
-      </c>
-      <c r="D27" s="13" t="s">
-        <v>53</v>
-      </c>
-      <c r="E27" s="13" t="s">
-        <v>196</v>
-      </c>
-      <c r="F27" s="13" t="s">
-        <v>197</v>
-      </c>
-      <c r="G27" s="13" t="s">
-        <v>198</v>
-      </c>
-      <c r="H27" s="13" t="s">
-        <v>199</v>
-      </c>
-      <c r="I27" s="13" t="s">
-        <v>200</v>
-      </c>
-      <c r="J27" s="14" t="s">
-        <v>49</v>
-      </c>
-      <c r="K27" s="13" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="28" customFormat="false" ht="102.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A28" s="13" t="s">
-        <v>201</v>
-      </c>
-      <c r="B28" s="13" t="s">
-        <v>27</v>
-      </c>
-      <c r="C28" s="13" t="s">
-        <v>202</v>
-      </c>
-      <c r="D28" s="13" t="s">
-        <v>53</v>
-      </c>
-      <c r="E28" s="13" t="s">
-        <v>203</v>
-      </c>
-      <c r="F28" s="13" t="s">
-        <v>204</v>
-      </c>
-      <c r="G28" s="13"/>
-      <c r="H28" s="13" t="s">
-        <v>205</v>
-      </c>
-      <c r="I28" s="13" t="s">
-        <v>200</v>
-      </c>
-      <c r="J28" s="14" t="s">
-        <v>49</v>
-      </c>
-      <c r="K28" s="13" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="29" customFormat="false" ht="102.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A29" s="13" t="s">
-        <v>206</v>
-      </c>
-      <c r="B29" s="13" t="s">
-        <v>27</v>
-      </c>
-      <c r="C29" s="13" t="s">
-        <v>207</v>
-      </c>
-      <c r="D29" s="13" t="s">
-        <v>53</v>
-      </c>
-      <c r="E29" s="13" t="s">
-        <v>208</v>
-      </c>
-      <c r="F29" s="13" t="s">
-        <v>209</v>
-      </c>
-      <c r="G29" s="13"/>
-      <c r="H29" s="13" t="s">
-        <v>210</v>
-      </c>
-      <c r="I29" s="13" t="s">
-        <v>200</v>
-      </c>
-      <c r="J29" s="14" t="s">
-        <v>49</v>
-      </c>
-      <c r="K29" s="13" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="30" customFormat="false" ht="113.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A30" s="13" t="s">
-        <v>211</v>
-      </c>
-      <c r="B30" s="13" t="s">
-        <v>28</v>
-      </c>
-      <c r="C30" s="13" t="s">
-        <v>212</v>
-      </c>
-      <c r="D30" s="13" t="s">
-        <v>53</v>
-      </c>
-      <c r="E30" s="13" t="s">
-        <v>213</v>
-      </c>
-      <c r="F30" s="13" t="s">
-        <v>214</v>
-      </c>
-      <c r="G30" s="13" t="s">
-        <v>215</v>
-      </c>
-      <c r="H30" s="13" t="s">
-        <v>216</v>
-      </c>
-      <c r="I30" s="13" t="s">
-        <v>57</v>
-      </c>
-      <c r="J30" s="14" t="s">
-        <v>49</v>
-      </c>
-      <c r="K30" s="13" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="31" customFormat="false" ht="79.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A31" s="13" t="s">
-        <v>217</v>
-      </c>
-      <c r="B31" s="13" t="s">
-        <v>28</v>
-      </c>
-      <c r="C31" s="13" t="s">
-        <v>218</v>
-      </c>
-      <c r="D31" s="13" t="s">
-        <v>74</v>
-      </c>
-      <c r="E31" s="13" t="s">
-        <v>219</v>
-      </c>
-      <c r="F31" s="13" t="s">
-        <v>220</v>
-      </c>
-      <c r="G31" s="13" t="s">
-        <v>221</v>
-      </c>
-      <c r="H31" s="13" t="s">
-        <v>222</v>
-      </c>
-      <c r="I31" s="13" t="s">
-        <v>57</v>
-      </c>
-      <c r="J31" s="14" t="s">
-        <v>49</v>
-      </c>
-      <c r="K31" s="13" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="32" customFormat="false" ht="79.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A32" s="13" t="s">
-        <v>223</v>
-      </c>
-      <c r="B32" s="13" t="s">
-        <v>28</v>
-      </c>
-      <c r="C32" s="13" t="s">
-        <v>224</v>
-      </c>
-      <c r="D32" s="13" t="s">
-        <v>53</v>
-      </c>
-      <c r="E32" s="13" t="s">
-        <v>225</v>
-      </c>
-      <c r="F32" s="13" t="s">
-        <v>226</v>
-      </c>
-      <c r="G32" s="13"/>
-      <c r="H32" s="13" t="s">
-        <v>227</v>
-      </c>
-      <c r="I32" s="13" t="s">
-        <v>57</v>
-      </c>
-      <c r="J32" s="14" t="s">
-        <v>49</v>
-      </c>
-      <c r="K32" s="13" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="33" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A33" s="13" t="s">
-        <v>228</v>
-      </c>
-      <c r="B33" s="13" t="s">
-        <v>28</v>
-      </c>
-      <c r="C33" s="13" t="s">
-        <v>229</v>
-      </c>
-      <c r="D33" s="13" t="s">
-        <v>74</v>
-      </c>
-      <c r="E33" s="13" t="s">
-        <v>230</v>
-      </c>
-      <c r="F33" s="13" t="s">
-        <v>231</v>
-      </c>
-      <c r="G33" s="13" t="s">
-        <v>232</v>
-      </c>
-      <c r="H33" s="13" t="s">
-        <v>233</v>
-      </c>
-      <c r="I33" s="13" t="s">
-        <v>57</v>
-      </c>
-      <c r="J33" s="15" t="s">
-        <v>64</v>
-      </c>
-      <c r="K33" s="13" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="34" customFormat="false" ht="79.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A34" s="13" t="s">
-        <v>234</v>
-      </c>
-      <c r="B34" s="13" t="s">
-        <v>29</v>
-      </c>
-      <c r="C34" s="13" t="s">
-        <v>235</v>
-      </c>
-      <c r="D34" s="13" t="s">
-        <v>53</v>
-      </c>
-      <c r="E34" s="13" t="s">
-        <v>236</v>
-      </c>
-      <c r="F34" s="13" t="s">
-        <v>237</v>
-      </c>
-      <c r="G34" s="13" t="s">
-        <v>238</v>
-      </c>
-      <c r="H34" s="13" t="s">
-        <v>239</v>
-      </c>
-      <c r="I34" s="13" t="s">
-        <v>115</v>
-      </c>
-      <c r="J34" s="14" t="s">
-        <v>49</v>
-      </c>
-      <c r="K34" s="13" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="35" customFormat="false" ht="124.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A35" s="13" t="s">
-        <v>240</v>
-      </c>
-      <c r="B35" s="13" t="s">
-        <v>29</v>
-      </c>
-      <c r="C35" s="13" t="s">
-        <v>241</v>
-      </c>
-      <c r="D35" s="13" t="s">
-        <v>74</v>
-      </c>
-      <c r="E35" s="13" t="s">
-        <v>242</v>
-      </c>
-      <c r="F35" s="13" t="s">
-        <v>243</v>
-      </c>
-      <c r="G35" s="13"/>
-      <c r="H35" s="13" t="s">
-        <v>244</v>
-      </c>
-      <c r="I35" s="13" t="s">
-        <v>48</v>
-      </c>
-      <c r="J35" s="14" t="s">
-        <v>49</v>
-      </c>
-      <c r="K35" s="13" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="36" customFormat="false" ht="102.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A36" s="13" t="s">
-        <v>245</v>
-      </c>
-      <c r="B36" s="13" t="s">
-        <v>29</v>
-      </c>
-      <c r="C36" s="13" t="s">
-        <v>246</v>
-      </c>
-      <c r="D36" s="13" t="s">
-        <v>74</v>
-      </c>
-      <c r="E36" s="13" t="s">
-        <v>247</v>
-      </c>
-      <c r="F36" s="13" t="s">
-        <v>248</v>
-      </c>
-      <c r="G36" s="13" t="s">
-        <v>249</v>
-      </c>
-      <c r="H36" s="13" t="s">
-        <v>250</v>
-      </c>
-      <c r="I36" s="13" t="s">
-        <v>57</v>
-      </c>
-      <c r="J36" s="14" t="s">
-        <v>49</v>
-      </c>
-      <c r="K36" s="13" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="37" customFormat="false" ht="79.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A37" s="13" t="s">
-        <v>251</v>
-      </c>
-      <c r="B37" s="13" t="s">
-        <v>30</v>
-      </c>
-      <c r="C37" s="13" t="s">
-        <v>252</v>
-      </c>
-      <c r="D37" s="13" t="s">
-        <v>74</v>
-      </c>
-      <c r="E37" s="13" t="s">
-        <v>253</v>
-      </c>
-      <c r="F37" s="13" t="s">
-        <v>254</v>
-      </c>
-      <c r="G37" s="13"/>
-      <c r="H37" s="13" t="s">
-        <v>255</v>
-      </c>
-      <c r="I37" s="13" t="s">
-        <v>57</v>
-      </c>
-      <c r="J37" s="14" t="s">
-        <v>49</v>
-      </c>
-      <c r="K37" s="13" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="38" customFormat="false" ht="102.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A38" s="13" t="s">
-        <v>256</v>
-      </c>
-      <c r="B38" s="13" t="s">
-        <v>30</v>
-      </c>
-      <c r="C38" s="13" t="s">
-        <v>257</v>
-      </c>
-      <c r="D38" s="13" t="s">
-        <v>74</v>
-      </c>
-      <c r="E38" s="13" t="s">
-        <v>258</v>
-      </c>
-      <c r="F38" s="13" t="s">
-        <v>259</v>
-      </c>
-      <c r="G38" s="13"/>
-      <c r="H38" s="13" t="s">
-        <v>260</v>
-      </c>
-      <c r="I38" s="13" t="s">
-        <v>57</v>
-      </c>
-      <c r="J38" s="15" t="s">
-        <v>64</v>
-      </c>
-      <c r="K38" s="13" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="39" customFormat="false" ht="91" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A39" s="13" t="s">
-        <v>261</v>
-      </c>
-      <c r="B39" s="13" t="s">
-        <v>31</v>
-      </c>
-      <c r="C39" s="13" t="s">
-        <v>262</v>
-      </c>
-      <c r="D39" s="13" t="s">
-        <v>67</v>
-      </c>
-      <c r="E39" s="13" t="s">
-        <v>263</v>
-      </c>
-      <c r="F39" s="13" t="s">
-        <v>264</v>
-      </c>
-      <c r="G39" s="13" t="s">
-        <v>265</v>
-      </c>
-      <c r="H39" s="13" t="s">
-        <v>266</v>
-      </c>
-      <c r="I39" s="13" t="s">
-        <v>57</v>
-      </c>
-      <c r="J39" s="14" t="s">
-        <v>49</v>
-      </c>
-      <c r="K39" s="13" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="40" customFormat="false" ht="91" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A40" s="13" t="s">
-        <v>267</v>
-      </c>
-      <c r="B40" s="13" t="s">
-        <v>31</v>
-      </c>
-      <c r="C40" s="13" t="s">
-        <v>268</v>
-      </c>
-      <c r="D40" s="13" t="s">
-        <v>74</v>
-      </c>
-      <c r="E40" s="13" t="s">
-        <v>269</v>
-      </c>
-      <c r="F40" s="13" t="s">
-        <v>270</v>
-      </c>
-      <c r="G40" s="13" t="s">
-        <v>271</v>
-      </c>
-      <c r="H40" s="13" t="s">
-        <v>272</v>
-      </c>
-      <c r="I40" s="13" t="s">
-        <v>57</v>
-      </c>
-      <c r="J40" s="14" t="s">
-        <v>49</v>
-      </c>
-      <c r="K40" s="13" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="41" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A41" s="13" t="s">
-        <v>273</v>
-      </c>
-      <c r="B41" s="13" t="s">
-        <v>32</v>
-      </c>
-      <c r="C41" s="13" t="s">
-        <v>274</v>
-      </c>
-      <c r="D41" s="13" t="s">
-        <v>74</v>
-      </c>
-      <c r="E41" s="13" t="s">
-        <v>275</v>
-      </c>
-      <c r="F41" s="13" t="s">
-        <v>276</v>
-      </c>
-      <c r="G41" s="13" t="s">
-        <v>277</v>
-      </c>
-      <c r="H41" s="13" t="s">
-        <v>278</v>
-      </c>
-      <c r="I41" s="13" t="s">
-        <v>57</v>
-      </c>
-      <c r="J41" s="14" t="s">
-        <v>49</v>
-      </c>
-      <c r="K41" s="13" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="42" customFormat="false" ht="102.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A42" s="13" t="s">
-        <v>279</v>
-      </c>
-      <c r="B42" s="13" t="s">
-        <v>32</v>
-      </c>
-      <c r="C42" s="13" t="s">
-        <v>280</v>
-      </c>
-      <c r="D42" s="13" t="s">
-        <v>74</v>
-      </c>
-      <c r="E42" s="13" t="s">
-        <v>281</v>
-      </c>
-      <c r="F42" s="13" t="s">
-        <v>282</v>
-      </c>
-      <c r="G42" s="13" t="s">
-        <v>283</v>
-      </c>
-      <c r="H42" s="13" t="s">
-        <v>284</v>
-      </c>
-      <c r="I42" s="13" t="s">
-        <v>285</v>
-      </c>
-      <c r="J42" s="14" t="s">
-        <v>49</v>
-      </c>
-      <c r="K42" s="13" t="s">
+      <c r="K42" s="14" t="s">
         <v>50</v>
       </c>
     </row>
@@ -3623,417 +3627,417 @@
   <dimension ref="A1:E24"/>
   <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="7"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="26"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="44"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="4" style="0" width="52"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="7"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="26"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="44"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="4" style="1" width="52"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="12" t="s">
+    <row r="1" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A1" s="13" t="s">
         <v>33</v>
       </c>
-      <c r="B1" s="12" t="s">
+      <c r="B1" s="13" t="s">
         <v>34</v>
       </c>
-      <c r="C1" s="12" t="s">
+      <c r="C1" s="13" t="s">
         <v>286</v>
       </c>
-      <c r="D1" s="12" t="s">
+      <c r="D1" s="13" t="s">
         <v>287</v>
       </c>
-      <c r="E1" s="12" t="s">
+      <c r="E1" s="13" t="s">
         <v>288</v>
       </c>
     </row>
-    <row r="2" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="13" t="s">
+    <row r="2" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A2" s="14" t="s">
         <v>289</v>
       </c>
-      <c r="B2" s="13" t="s">
+      <c r="B2" s="14" t="s">
         <v>17</v>
       </c>
-      <c r="C2" s="13" t="s">
+      <c r="C2" s="14" t="s">
         <v>290</v>
       </c>
-      <c r="D2" s="13" t="s">
+      <c r="D2" s="14" t="s">
         <v>291</v>
       </c>
-      <c r="E2" s="13" t="s">
+      <c r="E2" s="14" t="s">
         <v>292</v>
       </c>
     </row>
-    <row r="3" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="13" t="s">
+    <row r="3" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A3" s="14" t="s">
         <v>293</v>
       </c>
-      <c r="B3" s="13" t="s">
+      <c r="B3" s="14" t="s">
         <v>19</v>
       </c>
-      <c r="C3" s="13" t="s">
+      <c r="C3" s="14" t="s">
         <v>294</v>
       </c>
-      <c r="D3" s="13" t="s">
+      <c r="D3" s="14" t="s">
         <v>295</v>
       </c>
-      <c r="E3" s="13" t="s">
+      <c r="E3" s="14" t="s">
         <v>296</v>
       </c>
     </row>
-    <row r="4" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="13" t="s">
+    <row r="4" customFormat="false" ht="57" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A4" s="14" t="s">
         <v>297</v>
       </c>
-      <c r="B4" s="13" t="s">
+      <c r="B4" s="14" t="s">
         <v>21</v>
       </c>
-      <c r="C4" s="13" t="s">
+      <c r="C4" s="14" t="s">
         <v>298</v>
       </c>
-      <c r="D4" s="13" t="s">
+      <c r="D4" s="14" t="s">
         <v>299</v>
       </c>
-      <c r="E4" s="13" t="s">
+      <c r="E4" s="14" t="s">
         <v>300</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="13" t="s">
+    <row r="5" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A5" s="14" t="s">
         <v>301</v>
       </c>
-      <c r="B5" s="13" t="s">
+      <c r="B5" s="14" t="s">
         <v>21</v>
       </c>
-      <c r="C5" s="13" t="s">
+      <c r="C5" s="14" t="s">
         <v>302</v>
       </c>
-      <c r="D5" s="13" t="s">
+      <c r="D5" s="14" t="s">
         <v>303</v>
       </c>
-      <c r="E5" s="13" t="s">
+      <c r="E5" s="14" t="s">
         <v>304</v>
       </c>
     </row>
-    <row r="6" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="13" t="s">
+    <row r="6" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A6" s="14" t="s">
         <v>305</v>
       </c>
-      <c r="B6" s="13" t="s">
+      <c r="B6" s="14" t="s">
         <v>23</v>
       </c>
-      <c r="C6" s="13" t="s">
+      <c r="C6" s="14" t="s">
         <v>306</v>
       </c>
-      <c r="D6" s="13" t="s">
+      <c r="D6" s="14" t="s">
         <v>307</v>
       </c>
-      <c r="E6" s="13" t="s">
+      <c r="E6" s="14" t="s">
         <v>308</v>
       </c>
     </row>
-    <row r="7" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="13" t="s">
+    <row r="7" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A7" s="14" t="s">
         <v>309</v>
       </c>
-      <c r="B7" s="13" t="s">
+      <c r="B7" s="14" t="s">
         <v>26</v>
       </c>
-      <c r="C7" s="13" t="s">
+      <c r="C7" s="14" t="s">
         <v>310</v>
       </c>
-      <c r="D7" s="13" t="s">
+      <c r="D7" s="14" t="s">
         <v>311</v>
       </c>
-      <c r="E7" s="13" t="s">
+      <c r="E7" s="14" t="s">
         <v>312</v>
       </c>
     </row>
-    <row r="8" customFormat="false" ht="68.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="13" t="s">
+    <row r="8" customFormat="false" ht="68.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A8" s="14" t="s">
         <v>313</v>
       </c>
-      <c r="B8" s="13" t="s">
+      <c r="B8" s="14" t="s">
         <v>15</v>
       </c>
-      <c r="C8" s="13" t="s">
+      <c r="C8" s="14" t="s">
         <v>314</v>
       </c>
-      <c r="D8" s="13" t="s">
+      <c r="D8" s="14" t="s">
         <v>315</v>
       </c>
-      <c r="E8" s="13" t="s">
+      <c r="E8" s="14" t="s">
         <v>316</v>
       </c>
     </row>
-    <row r="9" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="13" t="s">
+    <row r="9" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A9" s="14" t="s">
         <v>317</v>
       </c>
-      <c r="B9" s="13" t="s">
+      <c r="B9" s="14" t="s">
         <v>15</v>
       </c>
-      <c r="C9" s="13" t="s">
+      <c r="C9" s="14" t="s">
         <v>318</v>
       </c>
-      <c r="D9" s="13" t="s">
+      <c r="D9" s="14" t="s">
         <v>319</v>
       </c>
-      <c r="E9" s="13" t="s">
+      <c r="E9" s="14" t="s">
         <v>320</v>
       </c>
     </row>
-    <row r="10" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="13" t="s">
+    <row r="10" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A10" s="14" t="s">
         <v>321</v>
       </c>
-      <c r="B10" s="13" t="s">
+      <c r="B10" s="14" t="s">
         <v>15</v>
       </c>
-      <c r="C10" s="13" t="s">
+      <c r="C10" s="14" t="s">
         <v>322</v>
       </c>
-      <c r="D10" s="13" t="s">
+      <c r="D10" s="14" t="s">
         <v>323</v>
       </c>
-      <c r="E10" s="13" t="s">
+      <c r="E10" s="14" t="s">
         <v>324</v>
       </c>
     </row>
-    <row r="11" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="13" t="s">
+    <row r="11" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A11" s="14" t="s">
         <v>325</v>
       </c>
-      <c r="B11" s="13" t="s">
+      <c r="B11" s="14" t="s">
         <v>28</v>
       </c>
-      <c r="C11" s="13" t="s">
+      <c r="C11" s="14" t="s">
         <v>326</v>
       </c>
-      <c r="D11" s="13" t="s">
+      <c r="D11" s="14" t="s">
         <v>327</v>
       </c>
-      <c r="E11" s="13" t="s">
+      <c r="E11" s="14" t="s">
         <v>328</v>
       </c>
     </row>
-    <row r="12" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="13" t="s">
+    <row r="12" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A12" s="14" t="s">
         <v>329</v>
       </c>
-      <c r="B12" s="13" t="s">
+      <c r="B12" s="14" t="s">
         <v>28</v>
       </c>
-      <c r="C12" s="13" t="s">
+      <c r="C12" s="14" t="s">
         <v>330</v>
       </c>
-      <c r="D12" s="13" t="s">
+      <c r="D12" s="14" t="s">
         <v>331</v>
       </c>
-      <c r="E12" s="13" t="s">
+      <c r="E12" s="14" t="s">
         <v>332</v>
       </c>
     </row>
-    <row r="13" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="13" t="s">
+    <row r="13" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A13" s="14" t="s">
         <v>333</v>
       </c>
-      <c r="B13" s="13" t="s">
+      <c r="B13" s="14" t="s">
         <v>28</v>
       </c>
-      <c r="C13" s="13" t="s">
+      <c r="C13" s="14" t="s">
         <v>334</v>
       </c>
-      <c r="D13" s="13" t="s">
+      <c r="D13" s="14" t="s">
         <v>335</v>
       </c>
-      <c r="E13" s="13" t="s">
+      <c r="E13" s="14" t="s">
         <v>336</v>
       </c>
     </row>
-    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="13" t="s">
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A14" s="14" t="s">
         <v>337</v>
       </c>
-      <c r="B14" s="13" t="s">
+      <c r="B14" s="14" t="s">
         <v>28</v>
       </c>
-      <c r="C14" s="13" t="s">
+      <c r="C14" s="14" t="s">
         <v>338</v>
       </c>
-      <c r="D14" s="13" t="s">
+      <c r="D14" s="14" t="s">
         <v>339</v>
       </c>
-      <c r="E14" s="13" t="s">
+      <c r="E14" s="14" t="s">
         <v>340</v>
       </c>
     </row>
-    <row r="15" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="13" t="s">
+    <row r="15" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A15" s="14" t="s">
         <v>341</v>
       </c>
-      <c r="B15" s="13" t="s">
+      <c r="B15" s="14" t="s">
         <v>31</v>
       </c>
-      <c r="C15" s="13" t="s">
+      <c r="C15" s="14" t="s">
         <v>342</v>
       </c>
-      <c r="D15" s="13" t="s">
+      <c r="D15" s="14" t="s">
         <v>343</v>
       </c>
-      <c r="E15" s="13" t="s">
+      <c r="E15" s="14" t="s">
         <v>344</v>
       </c>
     </row>
-    <row r="16" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="13" t="s">
+    <row r="16" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A16" s="14" t="s">
         <v>345</v>
       </c>
-      <c r="B16" s="13" t="s">
+      <c r="B16" s="14" t="s">
         <v>31</v>
       </c>
-      <c r="C16" s="13" t="s">
+      <c r="C16" s="14" t="s">
         <v>346</v>
       </c>
-      <c r="D16" s="13" t="s">
+      <c r="D16" s="14" t="s">
         <v>347</v>
       </c>
-      <c r="E16" s="13" t="s">
+      <c r="E16" s="14" t="s">
         <v>348</v>
       </c>
     </row>
-    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="13" t="s">
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A17" s="14" t="s">
         <v>349</v>
       </c>
-      <c r="B17" s="13" t="s">
+      <c r="B17" s="14" t="s">
         <v>31</v>
       </c>
-      <c r="C17" s="13" t="s">
+      <c r="C17" s="14" t="s">
         <v>350</v>
       </c>
-      <c r="D17" s="13" t="s">
+      <c r="D17" s="14" t="s">
         <v>351</v>
       </c>
-      <c r="E17" s="13" t="s">
+      <c r="E17" s="14" t="s">
         <v>352</v>
       </c>
     </row>
-    <row r="18" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="13" t="s">
+    <row r="18" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A18" s="14" t="s">
         <v>353</v>
       </c>
-      <c r="B18" s="13" t="s">
+      <c r="B18" s="14" t="s">
         <v>32</v>
       </c>
-      <c r="C18" s="13" t="s">
+      <c r="C18" s="14" t="s">
         <v>354</v>
       </c>
-      <c r="D18" s="13" t="s">
+      <c r="D18" s="14" t="s">
         <v>355</v>
       </c>
-      <c r="E18" s="13" t="s">
+      <c r="E18" s="14" t="s">
         <v>356</v>
       </c>
     </row>
-    <row r="19" customFormat="false" ht="68.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="13" t="s">
+    <row r="19" customFormat="false" ht="68.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A19" s="14" t="s">
         <v>357</v>
       </c>
-      <c r="B19" s="13" t="s">
+      <c r="B19" s="14" t="s">
         <v>32</v>
       </c>
-      <c r="C19" s="13" t="s">
+      <c r="C19" s="14" t="s">
         <v>358</v>
       </c>
-      <c r="D19" s="13" t="s">
+      <c r="D19" s="14" t="s">
         <v>359</v>
       </c>
-      <c r="E19" s="13" t="s">
+      <c r="E19" s="14" t="s">
         <v>360</v>
       </c>
     </row>
-    <row r="20" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="13" t="s">
+    <row r="20" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A20" s="14" t="s">
         <v>361</v>
       </c>
-      <c r="B20" s="13" t="s">
+      <c r="B20" s="14" t="s">
         <v>32</v>
       </c>
-      <c r="C20" s="13" t="s">
+      <c r="C20" s="14" t="s">
         <v>362</v>
       </c>
-      <c r="D20" s="13" t="s">
+      <c r="D20" s="14" t="s">
         <v>363</v>
       </c>
-      <c r="E20" s="13" t="s">
+      <c r="E20" s="14" t="s">
         <v>364</v>
       </c>
     </row>
-    <row r="21" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="13" t="s">
+    <row r="21" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A21" s="14" t="s">
         <v>365</v>
       </c>
-      <c r="B21" s="13" t="s">
+      <c r="B21" s="14" t="s">
         <v>32</v>
       </c>
-      <c r="C21" s="13" t="s">
+      <c r="C21" s="14" t="s">
         <v>366</v>
       </c>
-      <c r="D21" s="13" t="s">
+      <c r="D21" s="14" t="s">
         <v>367</v>
       </c>
-      <c r="E21" s="13" t="s">
+      <c r="E21" s="14" t="s">
         <v>368</v>
       </c>
     </row>
-    <row r="22" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="13" t="s">
+    <row r="22" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A22" s="14" t="s">
         <v>369</v>
       </c>
-      <c r="B22" s="13" t="s">
+      <c r="B22" s="14" t="s">
         <v>32</v>
       </c>
-      <c r="C22" s="13" t="s">
+      <c r="C22" s="14" t="s">
         <v>370</v>
       </c>
-      <c r="D22" s="13" t="s">
+      <c r="D22" s="14" t="s">
         <v>371</v>
       </c>
-      <c r="E22" s="13" t="s">
+      <c r="E22" s="14" t="s">
         <v>372</v>
       </c>
     </row>
-    <row r="23" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="13" t="s">
+    <row r="23" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A23" s="14" t="s">
         <v>373</v>
       </c>
-      <c r="B23" s="13" t="s">
+      <c r="B23" s="14" t="s">
         <v>374</v>
       </c>
-      <c r="C23" s="13" t="s">
+      <c r="C23" s="14" t="s">
         <v>375</v>
       </c>
-      <c r="D23" s="13" t="s">
+      <c r="D23" s="14" t="s">
         <v>376</v>
       </c>
-      <c r="E23" s="13" t="s">
+      <c r="E23" s="14" t="s">
         <v>377</v>
       </c>
     </row>
-    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="13" t="s">
+    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A24" s="14" t="s">
         <v>378</v>
       </c>
-      <c r="B24" s="13" t="s">
+      <c r="B24" s="14" t="s">
         <v>374</v>
       </c>
-      <c r="C24" s="13" t="s">
+      <c r="C24" s="14" t="s">
         <v>379</v>
       </c>
-      <c r="D24" s="13" t="s">
+      <c r="D24" s="14" t="s">
         <v>380</v>
       </c>
-      <c r="E24" s="13" t="s">
+      <c r="E24" s="14" t="s">
         <v>381</v>
       </c>
     </row>

</xml_diff>